<commit_message>
feat: add holiday-adjusted TTM, liquidity ranking and spread analysis
</commit_message>
<xml_diff>
--- a/usd-futures-curve-analyzer-matba-rofex/close.xlsx
+++ b/usd-futures-curve-analyzer-matba-rofex/close.xlsx
@@ -487,7 +487,7 @@
     <row r="6" ht="17.95" customHeight="1">
       <c s="4" t="inlineStr" r="A6">
         <is>
-          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : viernes, 10 de abril de 2026</t>
+          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : viernes, 17 de abril de 2026</t>
         </is>
       </c>
     </row>
@@ -690,34 +690,34 @@
         </is>
       </c>
       <c s="11" r="C11">
-        <v>1397.500000</v>
+        <v>1366.500000</v>
       </c>
       <c s="12" r="D11">
-        <v>1394.500000</v>
+        <v>1366.000000</v>
       </c>
       <c s="12" r="E11">
-        <v>1384.500000</v>
+        <v>1358.000000</v>
       </c>
       <c s="12" r="F11">
-        <v>1396.500000</v>
+        <v>1379.000000</v>
       </c>
       <c s="12" r="H11">
-        <v>1387.000000</v>
+        <v>1372.500000</v>
       </c>
       <c s="13" r="I11">
-        <v>892466.000000</v>
+        <v>982794.000000</v>
       </c>
       <c s="12" r="J11">
-        <v>1387.000000</v>
+        <v>1373.000000</v>
       </c>
       <c s="14" r="K11">
-        <v>-0.75</v>
+        <v>0.48</v>
       </c>
       <c s="13" r="L11">
-        <v>1486725.000000</v>
+        <v>1327955.000000</v>
       </c>
       <c s="13" r="M11">
-        <v>26688</v>
+        <v>-2255</v>
       </c>
       <c s="9" t="inlineStr" r="P11">
         <is>
@@ -730,13 +730,13 @@
         </is>
       </c>
       <c s="13" r="R11">
-        <v>150.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="S11">
-        <v>660.000000</v>
+        <v>940.000000</v>
       </c>
       <c s="13" r="T11">
-        <v>150000.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="8" t="str" r="U11"/>
       <c s="9" t="inlineStr" r="V11">
@@ -757,34 +757,34 @@
         </is>
       </c>
       <c s="11" r="C12">
-        <v>1422.000000</v>
+        <v>1387.000000</v>
       </c>
       <c s="12" r="D12">
-        <v>1420.000000</v>
+        <v>1383.000000</v>
       </c>
       <c s="12" r="E12">
-        <v>1407.000000</v>
+        <v>1378.000000</v>
       </c>
       <c s="12" r="F12">
-        <v>1420.000000</v>
+        <v>1398.500000</v>
       </c>
       <c s="12" r="H12">
-        <v>1410.500000</v>
+        <v>1394.000000</v>
       </c>
       <c s="13" r="I12">
-        <v>333535.000000</v>
+        <v>371341.000000</v>
       </c>
       <c s="12" r="J12">
-        <v>1410.000000</v>
+        <v>1394.000000</v>
       </c>
       <c s="14" r="K12">
-        <v>-0.84</v>
+        <v>0.50</v>
       </c>
       <c s="13" r="L12">
-        <v>2350127.000000</v>
+        <v>2383986.000000</v>
       </c>
       <c s="13" r="M12">
-        <v>24145</v>
+        <v>-28910</v>
       </c>
       <c s="9" t="inlineStr" r="P12">
         <is>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c s="13" r="R12">
-        <v>1462098.000000</v>
+        <v>1560084.000000</v>
       </c>
       <c s="13" r="S12">
-        <v>4621711.000000</v>
+        <v>4666149.000000</v>
       </c>
       <c s="13" r="T12">
-        <v>1462098000.000000</v>
+        <v>1560084000.000000</v>
       </c>
       <c s="8" t="str" r="U12"/>
       <c s="9" t="inlineStr" r="V12">
@@ -824,34 +824,34 @@
         </is>
       </c>
       <c s="11" r="C13">
-        <v>1452.000000</v>
+        <v>1414.000000</v>
       </c>
       <c s="12" r="D13">
-        <v>1448.000000</v>
+        <v>1409.500000</v>
       </c>
       <c s="12" r="E13">
-        <v>1436.500000</v>
+        <v>1406.000000</v>
       </c>
       <c s="12" r="F13">
-        <v>1448.500000</v>
+        <v>1425.000000</v>
       </c>
       <c s="12" r="H13">
-        <v>1438.000000</v>
+        <v>1421.000000</v>
       </c>
       <c s="13" r="I13">
-        <v>74622.000000</v>
+        <v>81396.000000</v>
       </c>
       <c s="12" r="J13">
-        <v>1439.000000</v>
+        <v>1420.500000</v>
       </c>
       <c s="14" r="K13">
-        <v>-0.90</v>
+        <v>0.46</v>
       </c>
       <c s="13" r="L13">
-        <v>272072.000000</v>
+        <v>319042.000000</v>
       </c>
       <c s="13" r="M13">
-        <v>19945</v>
+        <v>14894</v>
       </c>
       <c s="16" t="inlineStr" r="P13">
         <is>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c s="18" r="R13">
-        <v>1462248.000000</v>
+        <v>1560084.000000</v>
       </c>
       <c s="18" r="S13">
-        <v>4622371.000000</v>
+        <v>4667089.000000</v>
       </c>
       <c s="18" r="T13">
-        <v>1462248000.000000</v>
+        <v>1560084000.000000</v>
       </c>
       <c s="19" t="inlineStr" r="V13">
         <is>
@@ -890,34 +890,34 @@
         </is>
       </c>
       <c s="11" r="C14">
-        <v>1484.000000</v>
+        <v>1443.000000</v>
       </c>
       <c s="12" r="D14">
-        <v>1479.500000</v>
+        <v>1438.500000</v>
       </c>
       <c s="12" r="E14">
-        <v>1467.000000</v>
+        <v>1435.500000</v>
       </c>
       <c s="12" r="F14">
-        <v>1480.000000</v>
+        <v>1453.000000</v>
       </c>
       <c s="12" r="H14">
-        <v>1467.000000</v>
+        <v>1448.000000</v>
       </c>
       <c s="13" r="I14">
-        <v>16070.000000</v>
+        <v>45640.000000</v>
       </c>
       <c s="12" r="J14">
-        <v>1469.000000</v>
+        <v>1448.000000</v>
       </c>
       <c s="14" r="K14">
-        <v>-1.01</v>
+        <v>0.35</v>
       </c>
       <c s="13" r="L14">
-        <v>218581.000000</v>
+        <v>266763.000000</v>
       </c>
       <c s="13" r="M14">
-        <v>4901</v>
+        <v>10629</v>
       </c>
     </row>
     <row r="15" ht="14.15" customHeight="0">
@@ -932,34 +932,34 @@
         </is>
       </c>
       <c s="11" r="C15">
-        <v>1514.000000</v>
+        <v>1471.000000</v>
       </c>
       <c s="12" r="D15">
-        <v>1501.000000</v>
+        <v>1472.500000</v>
       </c>
       <c s="12" r="E15">
-        <v>1497.000000</v>
+        <v>1465.000000</v>
       </c>
       <c s="12" r="F15">
-        <v>1508.000000</v>
+        <v>1481.000000</v>
       </c>
       <c s="12" r="H15">
-        <v>1497.000000</v>
+        <v>1474.000000</v>
       </c>
       <c s="13" r="I15">
-        <v>11910.000000</v>
+        <v>22340.000000</v>
       </c>
       <c s="12" r="J15">
-        <v>1499.000000</v>
+        <v>1475.500000</v>
       </c>
       <c s="14" r="K15">
-        <v>-0.99</v>
+        <v>0.31</v>
       </c>
       <c s="13" r="L15">
-        <v>100154.000000</v>
+        <v>116778.000000</v>
       </c>
       <c s="13" r="M15">
-        <v>-1726</v>
+        <v>6176</v>
       </c>
     </row>
     <row r="16" ht="14.2" customHeight="0">
@@ -974,34 +974,34 @@
         </is>
       </c>
       <c s="11" r="C16">
-        <v>1547.000000</v>
+        <v>1500.000000</v>
       </c>
       <c s="12" r="D16">
-        <v>1543.000000</v>
+        <v>1496.000000</v>
       </c>
       <c s="12" r="E16">
-        <v>1529.500000</v>
+        <v>1490.000000</v>
       </c>
       <c s="12" r="F16">
-        <v>1543.000000</v>
+        <v>1513.000000</v>
       </c>
       <c s="12" r="H16">
-        <v>1529.500000</v>
+        <v>1505.000000</v>
       </c>
       <c s="13" r="I16">
-        <v>19233.000000</v>
+        <v>28564.000000</v>
       </c>
       <c s="12" r="J16">
-        <v>1530.000000</v>
+        <v>1504.000000</v>
       </c>
       <c s="14" r="K16">
-        <v>-1.10</v>
+        <v>0.27</v>
       </c>
       <c s="13" r="L16">
-        <v>56767.000000</v>
+        <v>83165.000000</v>
       </c>
       <c s="13" r="M16">
-        <v>-2664</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="17" ht="14.15" customHeight="0">
@@ -1016,34 +1016,34 @@
         </is>
       </c>
       <c s="11" r="C17">
-        <v>1580.000000</v>
+        <v>1530.500000</v>
       </c>
       <c s="12" r="D17">
-        <v>1565.000000</v>
+        <v>1515.500000</v>
       </c>
       <c s="12" r="E17">
-        <v>1565.000000</v>
+        <v>1515.500000</v>
       </c>
       <c s="12" r="F17">
-        <v>1570.000000</v>
+        <v>1535.500000</v>
       </c>
       <c s="12" r="H17">
-        <v>1566.500000</v>
+        <v>1530.000000</v>
       </c>
       <c s="13" r="I17">
-        <v>86961.000000</v>
+        <v>14338.000000</v>
       </c>
       <c s="12" r="J17">
-        <v>1564.000000</v>
+        <v>1531.500000</v>
       </c>
       <c s="14" r="K17">
-        <v>-1.01</v>
+        <v>0.07</v>
       </c>
       <c s="13" r="L17">
-        <v>75056.000000</v>
+        <v>88387.000000</v>
       </c>
       <c s="13" r="M17">
-        <v>22845</v>
+        <v>813</v>
       </c>
     </row>
     <row r="18" ht="14.2" customHeight="0">
@@ -1058,34 +1058,34 @@
         </is>
       </c>
       <c s="11" r="C18">
-        <v>1613.500000</v>
+        <v>1560.000000</v>
       </c>
       <c s="12" r="D18">
-        <v>1600.000000</v>
+        <v>1560.000000</v>
       </c>
       <c s="12" r="E18">
-        <v>1595.500000</v>
+        <v>1560.000000</v>
       </c>
       <c s="12" r="F18">
-        <v>1600.000000</v>
+        <v>1562.000000</v>
       </c>
       <c s="12" r="H18">
-        <v>1596.000000</v>
+        <v>1562.000000</v>
       </c>
       <c s="13" r="I18">
-        <v>26047.000000</v>
+        <v>210.000000</v>
       </c>
       <c s="12" r="J18">
-        <v>1596.500000</v>
+        <v>1562.000000</v>
       </c>
       <c s="14" r="K18">
-        <v>-1.05</v>
+        <v>0.13</v>
       </c>
       <c s="13" r="L18">
-        <v>39922.000000</v>
+        <v>47171.000000</v>
       </c>
       <c s="13" r="M18">
-        <v>7759</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="19" ht="14.15" customHeight="0">
@@ -1100,34 +1100,34 @@
         </is>
       </c>
       <c s="11" r="C19">
-        <v>1645.000000</v>
+        <v>1590.000000</v>
       </c>
       <c s="12" r="D19">
-        <v>1637.500000</v>
+        <v>1585.000000</v>
       </c>
       <c s="12" r="E19">
-        <v>1627.000000</v>
+        <v>1581.000000</v>
       </c>
       <c s="12" r="F19">
-        <v>1637.500000</v>
+        <v>1595.000000</v>
       </c>
       <c s="12" r="H19">
-        <v>1627.000000</v>
+        <v>1589.000000</v>
       </c>
       <c s="13" r="I19">
-        <v>1251.000000</v>
+        <v>13205.000000</v>
       </c>
       <c s="12" r="J19">
-        <v>1627.000000</v>
+        <v>1591.500000</v>
       </c>
       <c s="14" r="K19">
-        <v>-1.09</v>
+        <v>0.09</v>
       </c>
       <c s="13" r="L19">
-        <v>21218.000000</v>
+        <v>32004.000000</v>
       </c>
       <c s="13" r="M19">
-        <v>150</v>
+        <v>4486</v>
       </c>
     </row>
     <row r="20" ht="14.2" customHeight="0">
@@ -1142,31 +1142,31 @@
         </is>
       </c>
       <c s="11" r="C20">
-        <v>1679.000000</v>
+        <v>1623.000000</v>
       </c>
       <c s="12" r="D20">
-        <v>1670.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="E20">
-        <v>1670.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="F20">
-        <v>1673.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="H20">
-        <v>1673.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="I20">
-        <v>3.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="J20">
-        <v>1660.000000</v>
+        <v>1624.500000</v>
       </c>
       <c s="14" r="K20">
-        <v>-1.13</v>
+        <v>0.09</v>
       </c>
       <c s="13" r="L20">
-        <v>832.000000</v>
+        <v>807.000000</v>
       </c>
       <c s="13" r="M20">
         <v>0</v>
@@ -1184,242 +1184,207 @@
         </is>
       </c>
       <c s="11" r="C21">
-        <v>1709.000000</v>
+        <v>1653.000000</v>
       </c>
       <c s="12" r="D21">
-        <v>0.000000</v>
+        <v>1650.000000</v>
       </c>
       <c s="12" r="E21">
-        <v>0.000000</v>
+        <v>1650.000000</v>
       </c>
       <c s="12" r="F21">
-        <v>0.000000</v>
+        <v>1655.000000</v>
       </c>
       <c s="12" r="H21">
-        <v>0.000000</v>
+        <v>1653.500000</v>
       </c>
       <c s="13" r="I21">
-        <v>0.000000</v>
+        <v>256.000000</v>
       </c>
       <c s="12" r="J21">
-        <v>1690.000000</v>
+        <v>1655.000000</v>
       </c>
       <c s="14" r="K21">
-        <v>-1.11</v>
+        <v>0.12</v>
       </c>
       <c s="13" r="L21">
-        <v>257.000000</v>
+        <v>56.000000</v>
       </c>
       <c s="13" r="M21">
+        <v>-201</v>
+      </c>
+    </row>
+    <row r="22" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A22">
+        <is>
+          <t xml:space="preserve">DLR032027</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B22">
+        <is>
+          <t xml:space="preserve">31/3/2027</t>
+        </is>
+      </c>
+      <c s="11" r="C22">
+        <v>1680.000000</v>
+      </c>
+      <c s="12" r="D22">
+        <v>0.000000</v>
+      </c>
+      <c s="12" r="E22">
+        <v>0.000000</v>
+      </c>
+      <c s="12" r="F22">
+        <v>0.000000</v>
+      </c>
+      <c s="12" r="H22">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I22">
+        <v>0.000000</v>
+      </c>
+      <c s="12" r="J22">
+        <v>1685.000000</v>
+      </c>
+      <c s="14" r="K22">
+        <v>0.30</v>
+      </c>
+      <c s="13" r="L22">
+        <v>35.000000</v>
+      </c>
+      <c s="13" r="M22">
         <v>0</v>
       </c>
     </row>
-    <row r="22" ht="41.4" customHeight="1"/>
-    <row r="23" ht="14.15" customHeight="0">
-      <c s="5" t="inlineStr" r="A23">
+    <row r="23" ht="0.05" customHeight="1"/>
+    <row r="24" ht="41.4" customHeight="1"/>
+    <row r="25" ht="14.15" customHeight="0">
+      <c s="5" t="inlineStr" r="A25">
         <is>
           <t xml:space="preserve">Call</t>
         </is>
       </c>
-      <c s="5" t="inlineStr" r="B23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="H23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="I23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="J23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="K23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="L23">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="14.2" customHeight="0">
-      <c s="20" t="inlineStr" r="A24">
+      <c s="5" t="inlineStr" r="B25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="H25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="I25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="J25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="K25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="L25">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="14.2" customHeight="0">
+      <c s="20" t="inlineStr" r="A26">
         <is>
           <t xml:space="preserve">Posición</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="B24">
+      <c s="20" t="inlineStr" r="B26">
         <is>
           <t xml:space="preserve">Último Día Neg.</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="C24">
+      <c s="20" t="inlineStr" r="C26">
         <is>
           <t xml:space="preserve">Ejercicio</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="D24">
+      <c s="20" t="inlineStr" r="D26">
         <is>
           <t xml:space="preserve">Apertura</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="E24">
+      <c s="20" t="inlineStr" r="E26">
         <is>
           <t xml:space="preserve">Mín.</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="F24">
+      <c s="20" t="inlineStr" r="F26">
         <is>
           <t xml:space="preserve">Máx.</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="H24">
+      <c s="20" t="inlineStr" r="H26">
         <is>
           <t xml:space="preserve">Último</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="I24">
+      <c s="20" t="inlineStr" r="I26">
         <is>
           <t xml:space="preserve">Vol.</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="J24">
+      <c s="20" t="inlineStr" r="J26">
         <is>
           <t xml:space="preserve">Prima Ref. **</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="K24">
+      <c s="20" t="inlineStr" r="K26">
         <is>
           <t xml:space="preserve">I. A.*</t>
         </is>
       </c>
-      <c s="20" t="inlineStr" r="L24">
+      <c s="20" t="inlineStr" r="L26">
         <is>
           <t xml:space="preserve">Var. I.A.</t>
         </is>
-      </c>
-    </row>
-    <row r="25" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A25">
-        <is>
-          <t xml:space="preserve">DLR042026 Call 1400</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B25">
-        <is>
-          <t xml:space="preserve">30/4/2026</t>
-        </is>
-      </c>
-      <c s="21" r="C25">
-        <v>1400.0000</v>
-      </c>
-      <c s="22" r="D25">
-        <v>5.000000</v>
-      </c>
-      <c s="22" r="E25">
-        <v>5.000000</v>
-      </c>
-      <c s="22" r="F25">
-        <v>5.000000</v>
-      </c>
-      <c s="22" r="H25">
-        <v>5.000000</v>
-      </c>
-      <c s="13" r="I25">
-        <v>150.000000</v>
-      </c>
-      <c s="22" r="J25">
-        <v>9.933000</v>
-      </c>
-      <c s="13" r="K25">
-        <v>150.000000</v>
-      </c>
-      <c s="13" r="L25">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="26" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A26">
-        <is>
-          <t xml:space="preserve">DLR042026 Call 1430</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B26">
-        <is>
-          <t xml:space="preserve">30/4/2026</t>
-        </is>
-      </c>
-      <c s="21" r="C26">
-        <v>1430.0000</v>
-      </c>
-      <c s="22" r="D26">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="E26">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="F26">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="H26">
-        <v>0.000000</v>
-      </c>
-      <c s="13" r="I26">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="J26">
-        <v>2.807000</v>
-      </c>
-      <c s="13" r="K26">
-        <v>500.000000</v>
-      </c>
-      <c s="13" r="L26">
-        <v>0</v>
       </c>
     </row>
     <row r="27" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A27">
         <is>
-          <t xml:space="preserve">DLR052026 Call 1450</t>
+          <t xml:space="preserve">DLR042026 Call 1400</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B27">
         <is>
-          <t xml:space="preserve">29/5/2026</t>
+          <t xml:space="preserve">30/4/2026</t>
         </is>
       </c>
       <c s="21" r="C27">
-        <v>1450.0000</v>
+        <v>1400.0000</v>
       </c>
       <c s="22" r="D27">
         <v>0.000000</v>
@@ -1437,327 +1402,483 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J27">
-        <v>9.994000</v>
+        <v>3.375000</v>
       </c>
       <c s="13" r="K27">
-        <v>10.000000</v>
+        <v>150.000000</v>
       </c>
       <c s="13" r="L27">
         <v>0</v>
       </c>
     </row>
-    <row r="28" ht="14.15" customHeight="0">
-      <c s="6" t="inlineStr" r="A28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="B28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="H28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="I28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="J28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="K28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="L28">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="0.05" customHeight="1"/>
-    <row r="30" ht="28.35" customHeight="1"/>
-    <row r="31" ht="18" customHeight="0">
-      <c s="23" t="inlineStr" r="A31">
+    <row r="28" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A28">
+        <is>
+          <t xml:space="preserve">DLR042026 Call 1430</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B28">
+        <is>
+          <t xml:space="preserve">30/4/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C28">
+        <v>1430.0000</v>
+      </c>
+      <c s="22" r="D28">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E28">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F28">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H28">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I28">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J28">
+        <v>0.457000</v>
+      </c>
+      <c s="13" r="K28">
+        <v>500.000000</v>
+      </c>
+      <c s="13" r="L28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A29">
+        <is>
+          <t xml:space="preserve">DLR052026 Call 1400</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B29">
+        <is>
+          <t xml:space="preserve">29/5/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C29">
+        <v>1400.0000</v>
+      </c>
+      <c s="22" r="D29">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E29">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F29">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H29">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I29">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J29">
+        <v>19.645000</v>
+      </c>
+      <c s="13" r="K29">
+        <v>275.000000</v>
+      </c>
+      <c s="13" r="L29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A30">
+        <is>
+          <t xml:space="preserve">DLR052026 Call 1410</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B30">
+        <is>
+          <t xml:space="preserve">29/5/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C30">
+        <v>1410.0000</v>
+      </c>
+      <c s="22" r="D30">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E30">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F30">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H30">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I30">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J30">
+        <v>15.592000</v>
+      </c>
+      <c s="13" r="K30">
+        <v>5.000000</v>
+      </c>
+      <c s="13" r="L30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A31">
+        <is>
+          <t xml:space="preserve">DLR052026 Call 1450</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B31">
+        <is>
+          <t xml:space="preserve">29/5/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C31">
+        <v>1450.0000</v>
+      </c>
+      <c s="22" r="D31">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E31">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F31">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H31">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I31">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J31">
+        <v>5.229000</v>
+      </c>
+      <c s="13" r="K31">
+        <v>10.000000</v>
+      </c>
+      <c s="13" r="L31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="14.15" customHeight="0">
+      <c s="6" t="inlineStr" r="A32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="B32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="H32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="I32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="J32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="K32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="L32">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="0.05" customHeight="1"/>
+    <row r="34" ht="28.3" customHeight="1"/>
+    <row r="35" ht="18" customHeight="0">
+      <c s="23" t="inlineStr" r="A35">
         <is>
           <t xml:space="preserve">Cotizaciones Spot</t>
         </is>
       </c>
-      <c s="23" t="inlineStr" r="B31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="C31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="D31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="E31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="F31">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="0">
-      <c s="24" t="inlineStr" r="A32">
+      <c s="23" t="inlineStr" r="B35">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="C35">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="D35">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="E35">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="F35">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="0">
+      <c s="24" t="inlineStr" r="A36">
         <is>
           <t xml:space="preserve">Producto</t>
         </is>
       </c>
-      <c s="7" t="inlineStr" r="B32">
+      <c s="7" t="inlineStr" r="B36">
         <is>
           <t xml:space="preserve">Última</t>
         </is>
       </c>
-      <c s="8" t="str" r="C32"/>
-      <c s="7" t="inlineStr" r="D32">
+      <c s="8" t="str" r="C36"/>
+      <c s="7" t="inlineStr" r="D36">
         <is>
           <t xml:space="preserve">Anterior</t>
         </is>
       </c>
-      <c s="8" t="str" r="E32"/>
-      <c s="24" t="inlineStr" r="F32">
+      <c s="8" t="str" r="E36"/>
+      <c s="24" t="inlineStr" r="F36">
         <is>
           <t xml:space="preserve">Var.%</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="14.15" customHeight="0">
-      <c s="25" t="inlineStr" r="A33">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="7" t="inlineStr" r="B33">
+    <row r="37" ht="14.15" customHeight="0">
+      <c s="25" t="inlineStr" r="A37">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="7" t="inlineStr" r="B37">
         <is>
           <t xml:space="preserve">Fecha</t>
         </is>
       </c>
-      <c s="7" t="inlineStr" r="C33">
+      <c s="7" t="inlineStr" r="C37">
         <is>
           <t xml:space="preserve">Cotización</t>
         </is>
       </c>
-      <c s="7" t="inlineStr" r="D33">
+      <c s="7" t="inlineStr" r="D37">
         <is>
           <t xml:space="preserve">Fecha</t>
         </is>
       </c>
-      <c s="7" t="inlineStr" r="E33">
+      <c s="7" t="inlineStr" r="E37">
         <is>
           <t xml:space="preserve">Cotización</t>
         </is>
       </c>
-      <c s="25" t="inlineStr" r="F33">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A34">
-        <is>
-          <t xml:space="preserve">Yuan CNH</t>
-        </is>
-      </c>
-      <c s="26" r="B34">
-        <v>46122</v>
-      </c>
-      <c s="11" r="C34">
-        <v>201.278000</v>
-      </c>
-      <c s="26" r="D34">
-        <v>46121</v>
-      </c>
-      <c s="11" r="E34">
-        <v>202.638600</v>
-      </c>
-      <c s="21" r="F34">
-        <v>-0.67144</v>
-      </c>
-    </row>
-    <row r="35" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A35">
-        <is>
-          <t xml:space="preserve">Dólar UST ART 000</t>
-        </is>
-      </c>
-      <c s="26" r="B35">
-        <v>46122</v>
-      </c>
-      <c s="11" r="C35">
-        <v>1370.000000</v>
-      </c>
-      <c s="26" r="D35">
-        <v>46121</v>
-      </c>
-      <c s="11" r="E35">
-        <v>1381.000000</v>
-      </c>
-      <c s="21" r="F35">
-        <v>-0.79652</v>
-      </c>
-    </row>
-    <row r="36" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A36">
-        <is>
-          <t xml:space="preserve">Euro</t>
-        </is>
-      </c>
-      <c s="26" r="B36">
-        <v>46122</v>
-      </c>
-      <c s="11" r="C36">
-        <v>1608.978000</v>
-      </c>
-      <c s="26" r="D36">
-        <v>46121</v>
-      </c>
-      <c s="11" r="E36">
-        <v>1616.306000</v>
-      </c>
-      <c s="21" r="F36">
-        <v>-0.45338</v>
-      </c>
-    </row>
-    <row r="37" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A37">
-        <is>
-          <t xml:space="preserve">Dólar BCRA A3500</t>
-        </is>
-      </c>
-      <c s="26" r="B37">
-        <v>46122</v>
-      </c>
-      <c s="11" r="C37">
-        <v>1373.903300</v>
-      </c>
-      <c s="26" r="D37">
-        <v>46121</v>
-      </c>
-      <c s="11" r="E37">
-        <v>1383.231200</v>
-      </c>
-      <c s="21" r="F37">
-        <v>-0.67436</v>
+      <c s="25" t="inlineStr" r="F37">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="38" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A38">
         <is>
+          <t xml:space="preserve">Dólar UST ART 000</t>
+        </is>
+      </c>
+      <c s="26" r="B38">
+        <v>46129</v>
+      </c>
+      <c s="11" r="C38">
+        <v>1364.500000</v>
+      </c>
+      <c s="26" r="D38">
+        <v>46128</v>
+      </c>
+      <c s="11" r="E38">
+        <v>1358.000000</v>
+      </c>
+      <c s="21" r="F38">
+        <v>0.47865</v>
+      </c>
+    </row>
+    <row r="39" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A39">
+        <is>
+          <t xml:space="preserve">Yuan CNH</t>
+        </is>
+      </c>
+      <c s="26" r="B39">
+        <v>46129</v>
+      </c>
+      <c s="11" r="C39">
+        <v>199.599400</v>
+      </c>
+      <c s="26" r="D39">
+        <v>46128</v>
+      </c>
+      <c s="11" r="E39">
+        <v>198.270400</v>
+      </c>
+      <c s="21" r="F39">
+        <v>0.67030</v>
+      </c>
+    </row>
+    <row r="40" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A40">
+        <is>
+          <t xml:space="preserve">Euro</t>
+        </is>
+      </c>
+      <c s="26" r="B40">
+        <v>46129</v>
+      </c>
+      <c s="11" r="C40">
+        <v>1604.428000</v>
+      </c>
+      <c s="26" r="D40">
+        <v>46128</v>
+      </c>
+      <c s="11" r="E40">
+        <v>1594.078000</v>
+      </c>
+      <c s="21" r="F40">
+        <v>0.64928</v>
+      </c>
+    </row>
+    <row r="41" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A41">
+        <is>
+          <t xml:space="preserve">Dólar BCRA A3500</t>
+        </is>
+      </c>
+      <c s="26" r="B41">
+        <v>46129</v>
+      </c>
+      <c s="11" r="C41">
+        <v>1360.030700</v>
+      </c>
+      <c s="26" r="D41">
+        <v>46128</v>
+      </c>
+      <c s="11" r="E41">
+        <v>1352.977400</v>
+      </c>
+      <c s="21" r="F41">
+        <v>0.52132</v>
+      </c>
+    </row>
+    <row r="42" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A42">
+        <is>
           <t xml:space="preserve">Dólar BNA</t>
         </is>
       </c>
-      <c s="26" r="B38">
-        <v>46122</v>
-      </c>
-      <c s="11" r="C38">
-        <v>1365.500000</v>
-      </c>
-      <c s="26" r="D38">
-        <v>46121</v>
-      </c>
-      <c s="11" r="E38">
-        <v>1376.500000</v>
-      </c>
-      <c s="21" r="F38">
-        <v>-0.79913</v>
-      </c>
-    </row>
-    <row r="39" ht="14.15" customHeight="0">
-      <c s="6" t="inlineStr" r="A39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="B39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F39">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="22.45" customHeight="1"/>
-    <row r="41" ht="18" customHeight="1">
-      <c s="27" t="inlineStr" r="A41">
+      <c s="26" r="B42">
+        <v>46129</v>
+      </c>
+      <c s="11" r="C42">
+        <v>1360.000000</v>
+      </c>
+      <c s="26" r="D42">
+        <v>46128</v>
+      </c>
+      <c s="11" r="E42">
+        <v>1353.500000</v>
+      </c>
+      <c s="21" r="F42">
+        <v>0.48024</v>
+      </c>
+    </row>
+    <row r="43" ht="14.15" customHeight="0">
+      <c s="6" t="inlineStr" r="A43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="B43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F43">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22.5" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1">
+      <c s="27" t="inlineStr" r="A45">
         <is>
           <t xml:space="preserve">* Los valores de interés abierto pueden variar una vez que se realice el proceso del día.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c s="27" t="inlineStr" r="A42">
+    <row r="46" ht="18" customHeight="1">
+      <c s="27" t="inlineStr" r="A46">
         <is>
           <t xml:space="preserve">** Los valores indicativos de las primas se calculan en base a los parámetros del SARP® y son valores teóricos. Los mismos no afectan el cálculo de márgenes y diferencias.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="17.95" customHeight="1">
-      <c s="27" t="inlineStr" r="A43">
+    <row r="47" ht="17.95" customHeight="1">
+      <c s="27" t="inlineStr" r="A47">
         <is>
           <t xml:space="preserve">Aquellas posiciones que registran volumen pero no tienen valores en "Apertura", "Mínimo", "Máximo" y "Último" fueron operadas a través de pases.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="0.05" customHeight="1"/>
+    <row r="48" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A2:S2"/>
@@ -1768,11 +1889,11 @@
     <mergeCell ref="T11:U11"/>
     <mergeCell ref="T12:U12"/>
     <mergeCell ref="T13:U13"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="A41:Y41"/>
-    <mergeCell ref="A42:Y42"/>
-    <mergeCell ref="A43:Y43"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="A45:Y45"/>
+    <mergeCell ref="A46:Y46"/>
+    <mergeCell ref="A47:Y47"/>
   </mergeCells>
   <pageMargins left="0.984251968503937" right="0.984251968503937" top="0.984251968503937" bottom="0.984251968503937" header="0.984251968503937" footer="0.984251968503937"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Refactor plotting, add contract formatter, and improve NS curve fitting
</commit_message>
<xml_diff>
--- a/usd-futures-curve-analyzer-matba-rofex/close.xlsx
+++ b/usd-futures-curve-analyzer-matba-rofex/close.xlsx
@@ -487,7 +487,7 @@
     <row r="6" ht="17.95" customHeight="1">
       <c s="4" t="inlineStr" r="A6">
         <is>
-          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : viernes, 17 de abril de 2026</t>
+          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : lunes, 27 de abril de 2026</t>
         </is>
       </c>
     </row>
@@ -690,34 +690,34 @@
         </is>
       </c>
       <c s="11" r="C11">
-        <v>1366.500000</v>
+        <v>1403.500000</v>
       </c>
       <c s="12" r="D11">
-        <v>1366.000000</v>
+        <v>1407.000000</v>
       </c>
       <c s="12" r="E11">
-        <v>1358.000000</v>
+        <v>1403.500000</v>
       </c>
       <c s="12" r="F11">
-        <v>1379.000000</v>
+        <v>1420.000000</v>
       </c>
       <c s="12" r="H11">
-        <v>1372.500000</v>
+        <v>1418.000000</v>
       </c>
       <c s="13" r="I11">
-        <v>982794.000000</v>
+        <v>1298190.000000</v>
       </c>
       <c s="12" r="J11">
-        <v>1373.000000</v>
+        <v>1417.500000</v>
       </c>
       <c s="14" r="K11">
-        <v>0.48</v>
+        <v>1.00</v>
       </c>
       <c s="13" r="L11">
-        <v>1327955.000000</v>
+        <v>1145541.000000</v>
       </c>
       <c s="13" r="M11">
-        <v>-2255</v>
+        <v>-98549</v>
       </c>
       <c s="9" t="inlineStr" r="P11">
         <is>
@@ -730,13 +730,13 @@
         </is>
       </c>
       <c s="13" r="R11">
-        <v>0.000000</v>
+        <v>950.000000</v>
       </c>
       <c s="13" r="S11">
-        <v>940.000000</v>
+        <v>1875.000000</v>
       </c>
       <c s="13" r="T11">
-        <v>0.000000</v>
+        <v>950000.000000</v>
       </c>
       <c s="8" t="str" r="U11"/>
       <c s="9" t="inlineStr" r="V11">
@@ -757,34 +757,34 @@
         </is>
       </c>
       <c s="11" r="C12">
-        <v>1387.000000</v>
+        <v>1426.000000</v>
       </c>
       <c s="12" r="D12">
-        <v>1383.000000</v>
+        <v>1429.000000</v>
       </c>
       <c s="12" r="E12">
-        <v>1378.000000</v>
+        <v>1429.000000</v>
       </c>
       <c s="12" r="F12">
-        <v>1398.500000</v>
+        <v>1441.000000</v>
       </c>
       <c s="12" r="H12">
-        <v>1394.000000</v>
+        <v>1438.500000</v>
       </c>
       <c s="13" r="I12">
-        <v>371341.000000</v>
+        <v>682930.000000</v>
       </c>
       <c s="12" r="J12">
-        <v>1394.000000</v>
+        <v>1438.500000</v>
       </c>
       <c s="14" r="K12">
-        <v>0.50</v>
+        <v>0.88</v>
       </c>
       <c s="13" r="L12">
-        <v>2383986.000000</v>
+        <v>2552338.000000</v>
       </c>
       <c s="13" r="M12">
-        <v>-28910</v>
+        <v>87643</v>
       </c>
       <c s="9" t="inlineStr" r="P12">
         <is>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c s="13" r="R12">
-        <v>1560084.000000</v>
+        <v>2437363.000000</v>
       </c>
       <c s="13" r="S12">
-        <v>4666149.000000</v>
+        <v>4953045.000000</v>
       </c>
       <c s="13" r="T12">
-        <v>1560084000.000000</v>
+        <v>2437363000.000000</v>
       </c>
       <c s="8" t="str" r="U12"/>
       <c s="9" t="inlineStr" r="V12">
@@ -824,34 +824,34 @@
         </is>
       </c>
       <c s="11" r="C13">
-        <v>1414.000000</v>
+        <v>1454.000000</v>
       </c>
       <c s="12" r="D13">
-        <v>1409.500000</v>
+        <v>1461.000000</v>
       </c>
       <c s="12" r="E13">
-        <v>1406.000000</v>
+        <v>1459.500000</v>
       </c>
       <c s="12" r="F13">
-        <v>1425.000000</v>
+        <v>1467.000000</v>
       </c>
       <c s="12" r="H13">
-        <v>1421.000000</v>
+        <v>1463.500000</v>
       </c>
       <c s="13" r="I13">
-        <v>81396.000000</v>
+        <v>306560.000000</v>
       </c>
       <c s="12" r="J13">
-        <v>1420.500000</v>
+        <v>1463.500000</v>
       </c>
       <c s="14" r="K13">
-        <v>0.46</v>
+        <v>0.65</v>
       </c>
       <c s="13" r="L13">
-        <v>319042.000000</v>
+        <v>534867.000000</v>
       </c>
       <c s="13" r="M13">
-        <v>14894</v>
+        <v>99085</v>
       </c>
       <c s="16" t="inlineStr" r="P13">
         <is>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c s="18" r="R13">
-        <v>1560084.000000</v>
+        <v>2438313.000000</v>
       </c>
       <c s="18" r="S13">
-        <v>4667089.000000</v>
+        <v>4954920.000000</v>
       </c>
       <c s="18" r="T13">
-        <v>1560084000.000000</v>
+        <v>2438313000.000000</v>
       </c>
       <c s="19" t="inlineStr" r="V13">
         <is>
@@ -890,34 +890,34 @@
         </is>
       </c>
       <c s="11" r="C14">
-        <v>1443.000000</v>
+        <v>1483.500000</v>
       </c>
       <c s="12" r="D14">
-        <v>1438.500000</v>
+        <v>1489.000000</v>
       </c>
       <c s="12" r="E14">
-        <v>1435.500000</v>
+        <v>1489.000000</v>
       </c>
       <c s="12" r="F14">
-        <v>1453.000000</v>
+        <v>1497.000000</v>
       </c>
       <c s="12" r="H14">
-        <v>1448.000000</v>
+        <v>1494.500000</v>
       </c>
       <c s="13" r="I14">
-        <v>45640.000000</v>
+        <v>97159.000000</v>
       </c>
       <c s="12" r="J14">
-        <v>1448.000000</v>
+        <v>1494.000000</v>
       </c>
       <c s="14" r="K14">
-        <v>0.35</v>
+        <v>0.71</v>
       </c>
       <c s="13" r="L14">
-        <v>266763.000000</v>
+        <v>358300.000000</v>
       </c>
       <c s="13" r="M14">
-        <v>10629</v>
+        <v>27932</v>
       </c>
     </row>
     <row r="15" ht="14.15" customHeight="0">
@@ -932,34 +932,34 @@
         </is>
       </c>
       <c s="11" r="C15">
-        <v>1471.000000</v>
+        <v>1511.500000</v>
       </c>
       <c s="12" r="D15">
-        <v>1472.500000</v>
+        <v>1515.000000</v>
       </c>
       <c s="12" r="E15">
-        <v>1465.000000</v>
+        <v>1515.000000</v>
       </c>
       <c s="12" r="F15">
-        <v>1481.000000</v>
+        <v>1528.000000</v>
       </c>
       <c s="12" r="H15">
-        <v>1474.000000</v>
+        <v>1522.000000</v>
       </c>
       <c s="13" r="I15">
-        <v>22340.000000</v>
+        <v>38633.000000</v>
       </c>
       <c s="12" r="J15">
-        <v>1475.500000</v>
+        <v>1524.500000</v>
       </c>
       <c s="14" r="K15">
-        <v>0.31</v>
+        <v>0.86</v>
       </c>
       <c s="13" r="L15">
-        <v>116778.000000</v>
+        <v>98990.000000</v>
       </c>
       <c s="13" r="M15">
-        <v>6176</v>
+        <v>-94</v>
       </c>
     </row>
     <row r="16" ht="14.2" customHeight="0">
@@ -974,34 +974,34 @@
         </is>
       </c>
       <c s="11" r="C16">
-        <v>1500.000000</v>
+        <v>1541.500000</v>
       </c>
       <c s="12" r="D16">
-        <v>1496.000000</v>
+        <v>1545.500000</v>
       </c>
       <c s="12" r="E16">
-        <v>1490.000000</v>
+        <v>1545.500000</v>
       </c>
       <c s="12" r="F16">
-        <v>1513.000000</v>
+        <v>1557.500000</v>
       </c>
       <c s="12" r="H16">
-        <v>1505.000000</v>
+        <v>1557.500000</v>
       </c>
       <c s="13" r="I16">
-        <v>28564.000000</v>
+        <v>8010.000000</v>
       </c>
       <c s="12" r="J16">
-        <v>1504.000000</v>
+        <v>1554.000000</v>
       </c>
       <c s="14" r="K16">
-        <v>0.27</v>
+        <v>0.81</v>
       </c>
       <c s="13" r="L16">
-        <v>83165.000000</v>
+        <v>81471.000000</v>
       </c>
       <c s="13" r="M16">
-        <v>4106</v>
+        <v>-2841</v>
       </c>
     </row>
     <row r="17" ht="14.15" customHeight="0">
@@ -1016,34 +1016,34 @@
         </is>
       </c>
       <c s="11" r="C17">
-        <v>1530.500000</v>
+        <v>1569.000000</v>
       </c>
       <c s="12" r="D17">
-        <v>1515.500000</v>
+        <v>1580.000000</v>
       </c>
       <c s="12" r="E17">
-        <v>1515.500000</v>
+        <v>1578.000000</v>
       </c>
       <c s="12" r="F17">
-        <v>1535.500000</v>
+        <v>1585.000000</v>
       </c>
       <c s="12" r="H17">
-        <v>1530.000000</v>
+        <v>1580.000000</v>
       </c>
       <c s="13" r="I17">
-        <v>14338.000000</v>
+        <v>1722.000000</v>
       </c>
       <c s="12" r="J17">
-        <v>1531.500000</v>
+        <v>1582.000000</v>
       </c>
       <c s="14" r="K17">
-        <v>0.07</v>
+        <v>0.83</v>
       </c>
       <c s="13" r="L17">
-        <v>88387.000000</v>
+        <v>91198.000000</v>
       </c>
       <c s="13" r="M17">
-        <v>813</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="18" ht="14.2" customHeight="0">
@@ -1058,34 +1058,34 @@
         </is>
       </c>
       <c s="11" r="C18">
-        <v>1560.000000</v>
+        <v>1598.000000</v>
       </c>
       <c s="12" r="D18">
-        <v>1560.000000</v>
+        <v>1608.000000</v>
       </c>
       <c s="12" r="E18">
-        <v>1560.000000</v>
+        <v>1605.000000</v>
       </c>
       <c s="12" r="F18">
-        <v>1562.000000</v>
+        <v>1615.000000</v>
       </c>
       <c s="12" r="H18">
-        <v>1562.000000</v>
+        <v>1609.000000</v>
       </c>
       <c s="13" r="I18">
-        <v>210.000000</v>
+        <v>381.000000</v>
       </c>
       <c s="12" r="J18">
-        <v>1562.000000</v>
+        <v>1610.000000</v>
       </c>
       <c s="14" r="K18">
-        <v>0.13</v>
+        <v>0.75</v>
       </c>
       <c s="13" r="L18">
-        <v>47171.000000</v>
+        <v>47422.000000</v>
       </c>
       <c s="13" r="M18">
-        <v>-200</v>
+        <v>-69</v>
       </c>
     </row>
     <row r="19" ht="14.15" customHeight="0">
@@ -1100,34 +1100,34 @@
         </is>
       </c>
       <c s="11" r="C19">
-        <v>1590.000000</v>
+        <v>1628.000000</v>
       </c>
       <c s="12" r="D19">
-        <v>1585.000000</v>
+        <v>1640.000000</v>
       </c>
       <c s="12" r="E19">
-        <v>1581.000000</v>
+        <v>1635.000000</v>
       </c>
       <c s="12" r="F19">
-        <v>1595.000000</v>
+        <v>1643.000000</v>
       </c>
       <c s="12" r="H19">
-        <v>1589.000000</v>
+        <v>1640.000000</v>
       </c>
       <c s="13" r="I19">
-        <v>13205.000000</v>
+        <v>2967.000000</v>
       </c>
       <c s="12" r="J19">
-        <v>1591.500000</v>
+        <v>1638.000000</v>
       </c>
       <c s="14" r="K19">
-        <v>0.09</v>
+        <v>0.61</v>
       </c>
       <c s="13" r="L19">
-        <v>32004.000000</v>
+        <v>40488.000000</v>
       </c>
       <c s="13" r="M19">
-        <v>4486</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="20" ht="14.2" customHeight="0">
@@ -1142,34 +1142,34 @@
         </is>
       </c>
       <c s="11" r="C20">
-        <v>1623.000000</v>
+        <v>1658.000000</v>
       </c>
       <c s="12" r="D20">
-        <v>0.000000</v>
+        <v>1675.000000</v>
       </c>
       <c s="12" r="E20">
-        <v>0.000000</v>
+        <v>1673.000000</v>
       </c>
       <c s="12" r="F20">
-        <v>0.000000</v>
+        <v>1675.000000</v>
       </c>
       <c s="12" r="H20">
-        <v>0.000000</v>
+        <v>1673.000000</v>
       </c>
       <c s="13" r="I20">
-        <v>0.000000</v>
+        <v>281.000000</v>
       </c>
       <c s="12" r="J20">
-        <v>1624.500000</v>
+        <v>1668.000000</v>
       </c>
       <c s="14" r="K20">
-        <v>0.09</v>
+        <v>0.60</v>
       </c>
       <c s="13" r="L20">
-        <v>807.000000</v>
+        <v>1205.000000</v>
       </c>
       <c s="13" r="M20">
-        <v>0</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" ht="14.15" customHeight="0">
@@ -1184,34 +1184,34 @@
         </is>
       </c>
       <c s="11" r="C21">
-        <v>1653.000000</v>
+        <v>1688.000000</v>
       </c>
       <c s="12" r="D21">
-        <v>1650.000000</v>
+        <v>1685.500000</v>
       </c>
       <c s="12" r="E21">
-        <v>1650.000000</v>
+        <v>1685.500000</v>
       </c>
       <c s="12" r="F21">
-        <v>1655.000000</v>
+        <v>1685.500000</v>
       </c>
       <c s="12" r="H21">
-        <v>1653.500000</v>
+        <v>1685.500000</v>
       </c>
       <c s="13" r="I21">
-        <v>256.000000</v>
+        <v>400.000000</v>
       </c>
       <c s="12" r="J21">
-        <v>1655.000000</v>
+        <v>1698.000000</v>
       </c>
       <c s="14" r="K21">
-        <v>0.12</v>
+        <v>0.59</v>
       </c>
       <c s="13" r="L21">
-        <v>56.000000</v>
+        <v>739.000000</v>
       </c>
       <c s="13" r="M21">
-        <v>-201</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22" ht="14.15" customHeight="0">
@@ -1226,34 +1226,34 @@
         </is>
       </c>
       <c s="11" r="C22">
-        <v>1680.000000</v>
+        <v>1716.000000</v>
       </c>
       <c s="12" r="D22">
-        <v>0.000000</v>
+        <v>1720.000000</v>
       </c>
       <c s="12" r="E22">
-        <v>0.000000</v>
+        <v>1720.000000</v>
       </c>
       <c s="12" r="F22">
-        <v>0.000000</v>
+        <v>1730.000000</v>
       </c>
       <c s="12" r="H22">
-        <v>0.000000</v>
+        <v>1730.000000</v>
       </c>
       <c s="13" r="I22">
-        <v>0.000000</v>
+        <v>130.000000</v>
       </c>
       <c s="12" r="J22">
-        <v>1685.000000</v>
+        <v>1730.000000</v>
       </c>
       <c s="14" r="K22">
-        <v>0.30</v>
+        <v>0.82</v>
       </c>
       <c s="13" r="L22">
-        <v>35.000000</v>
+        <v>486.000000</v>
       </c>
       <c s="13" r="M22">
-        <v>0</v>
+        <v>-30</v>
       </c>
     </row>
     <row r="23" ht="0.05" customHeight="1"/>
@@ -1402,7 +1402,7 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J27">
-        <v>3.375000</v>
+        <v>19.142000</v>
       </c>
       <c s="13" r="K27">
         <v>150.000000</v>
@@ -1441,7 +1441,7 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J28">
-        <v>0.457000</v>
+        <v>2.791000</v>
       </c>
       <c s="13" r="K28">
         <v>500.000000</v>
@@ -1480,7 +1480,7 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J29">
-        <v>19.645000</v>
+        <v>44.652000</v>
       </c>
       <c s="13" r="K29">
         <v>275.000000</v>
@@ -1492,7 +1492,7 @@
     <row r="30" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A30">
         <is>
-          <t xml:space="preserve">DLR052026 Call 1410</t>
+          <t xml:space="preserve">DLR052026 Call 1450</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B30">
@@ -1501,37 +1501,37 @@
         </is>
       </c>
       <c s="21" r="C30">
-        <v>1410.0000</v>
+        <v>1450.0000</v>
       </c>
       <c s="22" r="D30">
-        <v>0.000000</v>
+        <v>12.000000</v>
       </c>
       <c s="22" r="E30">
-        <v>0.000000</v>
+        <v>12.000000</v>
       </c>
       <c s="22" r="F30">
-        <v>0.000000</v>
+        <v>12.000000</v>
       </c>
       <c s="22" r="H30">
-        <v>0.000000</v>
+        <v>12.000000</v>
       </c>
       <c s="13" r="I30">
-        <v>0.000000</v>
+        <v>450.000000</v>
       </c>
       <c s="22" r="J30">
-        <v>15.592000</v>
+        <v>15.742000</v>
       </c>
       <c s="13" r="K30">
-        <v>5.000000</v>
+        <v>450.000000</v>
       </c>
       <c s="13" r="L30">
-        <v>0</v>
+        <v>450</v>
       </c>
     </row>
     <row r="31" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A31">
         <is>
-          <t xml:space="preserve">DLR052026 Call 1450</t>
+          <t xml:space="preserve">DLR052026 Call 1460</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B31">
@@ -1540,31 +1540,31 @@
         </is>
       </c>
       <c s="21" r="C31">
-        <v>1450.0000</v>
+        <v>1460.0000</v>
       </c>
       <c s="22" r="D31">
-        <v>0.000000</v>
+        <v>8.000000</v>
       </c>
       <c s="22" r="E31">
-        <v>0.000000</v>
+        <v>8.000000</v>
       </c>
       <c s="22" r="F31">
-        <v>0.000000</v>
+        <v>8.000000</v>
       </c>
       <c s="22" r="H31">
-        <v>0.000000</v>
+        <v>8.000000</v>
       </c>
       <c s="13" r="I31">
-        <v>0.000000</v>
+        <v>500.000000</v>
       </c>
       <c s="22" r="J31">
-        <v>5.229000</v>
+        <v>12.098000</v>
       </c>
       <c s="13" r="K31">
-        <v>10.000000</v>
+        <v>500.000000</v>
       </c>
       <c s="13" r="L31">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32" ht="14.15" customHeight="0">
@@ -1721,107 +1721,107 @@
         </is>
       </c>
       <c s="26" r="B38">
-        <v>46129</v>
+        <v>46139</v>
       </c>
       <c s="11" r="C38">
-        <v>1364.500000</v>
+        <v>1417.000000</v>
       </c>
       <c s="26" r="D38">
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c s="11" r="E38">
-        <v>1358.000000</v>
+        <v>1399.500000</v>
       </c>
       <c s="21" r="F38">
-        <v>0.47865</v>
+        <v>1.25045</v>
       </c>
     </row>
     <row r="39" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A39">
         <is>
-          <t xml:space="preserve">Yuan CNH</t>
+          <t xml:space="preserve">Dólar BCRA A3500</t>
         </is>
       </c>
       <c s="26" r="B39">
-        <v>46129</v>
+        <v>46139</v>
       </c>
       <c s="11" r="C39">
-        <v>199.599400</v>
+        <v>1412.986500</v>
       </c>
       <c s="26" r="D39">
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c s="11" r="E39">
-        <v>198.270400</v>
+        <v>1397.206300</v>
       </c>
       <c s="21" r="F39">
-        <v>0.67030</v>
+        <v>1.12941</v>
       </c>
     </row>
     <row r="40" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A40">
         <is>
-          <t xml:space="preserve">Euro</t>
+          <t xml:space="preserve">Yuan CNH</t>
         </is>
       </c>
       <c s="26" r="B40">
-        <v>46129</v>
+        <v>46139</v>
       </c>
       <c s="11" r="C40">
-        <v>1604.428000</v>
+        <v>206.970300</v>
       </c>
       <c s="26" r="D40">
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c s="11" r="E40">
-        <v>1594.078000</v>
+        <v>204.455300</v>
       </c>
       <c s="21" r="F40">
-        <v>0.64928</v>
+        <v>1.23010</v>
       </c>
     </row>
     <row r="41" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A41">
         <is>
-          <t xml:space="preserve">Dólar BCRA A3500</t>
+          <t xml:space="preserve">Dólar BNA</t>
         </is>
       </c>
       <c s="26" r="B41">
-        <v>46129</v>
+        <v>46139</v>
       </c>
       <c s="11" r="C41">
-        <v>1360.030700</v>
+        <v>1412.500000</v>
       </c>
       <c s="26" r="D41">
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c s="11" r="E41">
-        <v>1352.977400</v>
+        <v>1395.000000</v>
       </c>
       <c s="21" r="F41">
-        <v>0.52132</v>
+        <v>1.25448</v>
       </c>
     </row>
     <row r="42" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A42">
         <is>
-          <t xml:space="preserve">Dólar BNA</t>
+          <t xml:space="preserve">Euro</t>
         </is>
       </c>
       <c s="26" r="B42">
-        <v>46129</v>
+        <v>46139</v>
       </c>
       <c s="11" r="C42">
-        <v>1360.000000</v>
+        <v>1660.118000</v>
       </c>
       <c s="26" r="D42">
-        <v>46128</v>
+        <v>46136</v>
       </c>
       <c s="11" r="E42">
-        <v>1353.500000</v>
+        <v>1636.408000</v>
       </c>
       <c s="21" r="F42">
-        <v>0.48024</v>
+        <v>1.44891</v>
       </c>
     </row>
     <row r="43" ht="14.15" customHeight="0">

</xml_diff>

<commit_message>
fix: exclude expired contract (TTM=0) from curve to prevent spline error
</commit_message>
<xml_diff>
--- a/usd-futures-curve-analyzer-matba-rofex/close.xlsx
+++ b/usd-futures-curve-analyzer-matba-rofex/close.xlsx
@@ -487,7 +487,7 @@
     <row r="6" ht="17.95" customHeight="1">
       <c s="4" t="inlineStr" r="A6">
         <is>
-          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : lunes, 27 de abril de 2026</t>
+          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : jueves, 30 de abril de 2026</t>
         </is>
       </c>
     </row>
@@ -690,34 +690,34 @@
         </is>
       </c>
       <c s="11" r="C11">
-        <v>1403.500000</v>
+        <v>1391.500000</v>
       </c>
       <c s="12" r="D11">
-        <v>1407.000000</v>
+        <v>1390.000000</v>
       </c>
       <c s="12" r="E11">
-        <v>1403.500000</v>
+        <v>1377.000000</v>
       </c>
       <c s="12" r="F11">
-        <v>1420.000000</v>
+        <v>1390.000000</v>
       </c>
       <c s="12" r="H11">
-        <v>1418.000000</v>
+        <v>1381.000000</v>
       </c>
       <c s="13" r="I11">
-        <v>1298190.000000</v>
+        <v>880372.000000</v>
       </c>
       <c s="12" r="J11">
-        <v>1417.500000</v>
+        <v>1381.095400</v>
       </c>
       <c s="14" r="K11">
-        <v>1.00</v>
+        <v>-0.75</v>
       </c>
       <c s="13" r="L11">
-        <v>1145541.000000</v>
+        <v>879270.000000</v>
       </c>
       <c s="13" r="M11">
-        <v>-98549</v>
+        <v>-24712</v>
       </c>
       <c s="9" t="inlineStr" r="P11">
         <is>
@@ -730,13 +730,13 @@
         </is>
       </c>
       <c s="13" r="R11">
-        <v>950.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="S11">
-        <v>1875.000000</v>
+        <v>1726.000000</v>
       </c>
       <c s="13" r="T11">
-        <v>950000.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="8" t="str" r="U11"/>
       <c s="9" t="inlineStr" r="V11">
@@ -757,34 +757,34 @@
         </is>
       </c>
       <c s="11" r="C12">
-        <v>1426.000000</v>
+        <v>1413.500000</v>
       </c>
       <c s="12" r="D12">
-        <v>1429.000000</v>
+        <v>1409.000000</v>
       </c>
       <c s="12" r="E12">
-        <v>1429.000000</v>
+        <v>1402.000000</v>
       </c>
       <c s="12" r="F12">
-        <v>1441.000000</v>
+        <v>1418.500000</v>
       </c>
       <c s="12" r="H12">
-        <v>1438.500000</v>
+        <v>1415.500000</v>
       </c>
       <c s="13" r="I12">
-        <v>682930.000000</v>
+        <v>822988.000000</v>
       </c>
       <c s="12" r="J12">
-        <v>1438.500000</v>
+        <v>1416.000000</v>
       </c>
       <c s="14" r="K12">
-        <v>0.88</v>
+        <v>0.18</v>
       </c>
       <c s="13" r="L12">
-        <v>2552338.000000</v>
+        <v>2939947.000000</v>
       </c>
       <c s="13" r="M12">
-        <v>87643</v>
+        <v>81820</v>
       </c>
       <c s="9" t="inlineStr" r="P12">
         <is>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c s="13" r="R12">
-        <v>2437363.000000</v>
+        <v>1974201.000000</v>
       </c>
       <c s="13" r="S12">
-        <v>4953045.000000</v>
+        <v>5199984.000000</v>
       </c>
       <c s="13" r="T12">
-        <v>2437363000.000000</v>
+        <v>1974201000.000000</v>
       </c>
       <c s="8" t="str" r="U12"/>
       <c s="9" t="inlineStr" r="V12">
@@ -824,34 +824,34 @@
         </is>
       </c>
       <c s="11" r="C13">
-        <v>1454.000000</v>
+        <v>1440.000000</v>
       </c>
       <c s="12" r="D13">
-        <v>1461.000000</v>
+        <v>1434.000000</v>
       </c>
       <c s="12" r="E13">
-        <v>1459.500000</v>
+        <v>1428.000000</v>
       </c>
       <c s="12" r="F13">
-        <v>1467.000000</v>
+        <v>1447.000000</v>
       </c>
       <c s="12" r="H13">
-        <v>1463.500000</v>
+        <v>1443.000000</v>
       </c>
       <c s="13" r="I13">
-        <v>306560.000000</v>
+        <v>190696.000000</v>
       </c>
       <c s="12" r="J13">
-        <v>1463.500000</v>
+        <v>1443.500000</v>
       </c>
       <c s="14" r="K13">
-        <v>0.65</v>
+        <v>0.24</v>
       </c>
       <c s="13" r="L13">
-        <v>534867.000000</v>
+        <v>592327.000000</v>
       </c>
       <c s="13" r="M13">
-        <v>99085</v>
+        <v>26153</v>
       </c>
       <c s="16" t="inlineStr" r="P13">
         <is>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c s="18" r="R13">
-        <v>2438313.000000</v>
+        <v>1974201.000000</v>
       </c>
       <c s="18" r="S13">
-        <v>4954920.000000</v>
+        <v>5201710.000000</v>
       </c>
       <c s="18" r="T13">
-        <v>2438313000.000000</v>
+        <v>1974201000.000000</v>
       </c>
       <c s="19" t="inlineStr" r="V13">
         <is>
@@ -890,34 +890,34 @@
         </is>
       </c>
       <c s="11" r="C14">
-        <v>1483.500000</v>
+        <v>1470.000000</v>
       </c>
       <c s="12" r="D14">
-        <v>1489.000000</v>
+        <v>1461.500000</v>
       </c>
       <c s="12" r="E14">
-        <v>1489.000000</v>
+        <v>1458.500000</v>
       </c>
       <c s="12" r="F14">
-        <v>1497.000000</v>
+        <v>1476.500000</v>
       </c>
       <c s="12" r="H14">
-        <v>1494.500000</v>
+        <v>1470.500000</v>
       </c>
       <c s="13" r="I14">
-        <v>97159.000000</v>
+        <v>54466.000000</v>
       </c>
       <c s="12" r="J14">
-        <v>1494.000000</v>
+        <v>1474.000000</v>
       </c>
       <c s="14" r="K14">
-        <v>0.71</v>
+        <v>0.27</v>
       </c>
       <c s="13" r="L14">
-        <v>358300.000000</v>
+        <v>408191.000000</v>
       </c>
       <c s="13" r="M14">
-        <v>27932</v>
+        <v>6609</v>
       </c>
     </row>
     <row r="15" ht="14.15" customHeight="0">
@@ -932,34 +932,34 @@
         </is>
       </c>
       <c s="11" r="C15">
-        <v>1511.500000</v>
+        <v>1499.500000</v>
       </c>
       <c s="12" r="D15">
-        <v>1515.000000</v>
+        <v>1490.000000</v>
       </c>
       <c s="12" r="E15">
-        <v>1515.000000</v>
+        <v>1489.000000</v>
       </c>
       <c s="12" r="F15">
-        <v>1528.000000</v>
+        <v>1505.500000</v>
       </c>
       <c s="12" r="H15">
-        <v>1522.000000</v>
+        <v>1501.000000</v>
       </c>
       <c s="13" r="I15">
-        <v>38633.000000</v>
+        <v>2273.000000</v>
       </c>
       <c s="12" r="J15">
-        <v>1524.500000</v>
+        <v>1504.000000</v>
       </c>
       <c s="14" r="K15">
-        <v>0.86</v>
+        <v>0.30</v>
       </c>
       <c s="13" r="L15">
-        <v>98990.000000</v>
+        <v>106974.000000</v>
       </c>
       <c s="13" r="M15">
-        <v>-94</v>
+        <v>2241</v>
       </c>
     </row>
     <row r="16" ht="14.2" customHeight="0">
@@ -974,34 +974,34 @@
         </is>
       </c>
       <c s="11" r="C16">
-        <v>1541.500000</v>
+        <v>1530.000000</v>
       </c>
       <c s="12" r="D16">
-        <v>1545.500000</v>
+        <v>1520.000000</v>
       </c>
       <c s="12" r="E16">
-        <v>1545.500000</v>
+        <v>1520.000000</v>
       </c>
       <c s="12" r="F16">
-        <v>1557.500000</v>
+        <v>1552.000000</v>
       </c>
       <c s="12" r="H16">
-        <v>1557.500000</v>
+        <v>1535.000000</v>
       </c>
       <c s="13" r="I16">
-        <v>8010.000000</v>
+        <v>7258.000000</v>
       </c>
       <c s="12" r="J16">
-        <v>1554.000000</v>
+        <v>1535.000000</v>
       </c>
       <c s="14" r="K16">
-        <v>0.81</v>
+        <v>0.33</v>
       </c>
       <c s="13" r="L16">
-        <v>81471.000000</v>
+        <v>79122.000000</v>
       </c>
       <c s="13" r="M16">
-        <v>-2841</v>
+        <v>-330</v>
       </c>
     </row>
     <row r="17" ht="14.15" customHeight="0">
@@ -1016,34 +1016,34 @@
         </is>
       </c>
       <c s="11" r="C17">
-        <v>1569.000000</v>
+        <v>1560.000000</v>
       </c>
       <c s="12" r="D17">
-        <v>1580.000000</v>
+        <v>1550.000000</v>
       </c>
       <c s="12" r="E17">
-        <v>1578.000000</v>
+        <v>1550.000000</v>
       </c>
       <c s="12" r="F17">
-        <v>1585.000000</v>
+        <v>1564.500000</v>
       </c>
       <c s="12" r="H17">
-        <v>1580.000000</v>
+        <v>1564.500000</v>
       </c>
       <c s="13" r="I17">
-        <v>1722.000000</v>
+        <v>4549.000000</v>
       </c>
       <c s="12" r="J17">
-        <v>1582.000000</v>
+        <v>1564.500000</v>
       </c>
       <c s="14" r="K17">
-        <v>0.83</v>
+        <v>0.29</v>
       </c>
       <c s="13" r="L17">
-        <v>91198.000000</v>
+        <v>96152.000000</v>
       </c>
       <c s="13" r="M17">
-        <v>1276</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="18" ht="14.2" customHeight="0">
@@ -1058,34 +1058,34 @@
         </is>
       </c>
       <c s="11" r="C18">
-        <v>1598.000000</v>
+        <v>1589.000000</v>
       </c>
       <c s="12" r="D18">
-        <v>1608.000000</v>
+        <v>1590.000000</v>
       </c>
       <c s="12" r="E18">
-        <v>1605.000000</v>
+        <v>1590.000000</v>
       </c>
       <c s="12" r="F18">
-        <v>1615.000000</v>
+        <v>1600.000000</v>
       </c>
       <c s="12" r="H18">
-        <v>1609.000000</v>
+        <v>1600.000000</v>
       </c>
       <c s="13" r="I18">
-        <v>381.000000</v>
+        <v>2.000000</v>
       </c>
       <c s="12" r="J18">
-        <v>1610.000000</v>
+        <v>1594.500000</v>
       </c>
       <c s="14" r="K18">
-        <v>0.75</v>
+        <v>0.35</v>
       </c>
       <c s="13" r="L18">
-        <v>47422.000000</v>
+        <v>47385.000000</v>
       </c>
       <c s="13" r="M18">
-        <v>-69</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="19" ht="14.15" customHeight="0">
@@ -1100,34 +1100,34 @@
         </is>
       </c>
       <c s="11" r="C19">
-        <v>1628.000000</v>
+        <v>1619.000000</v>
       </c>
       <c s="12" r="D19">
-        <v>1640.000000</v>
+        <v>1600.000000</v>
       </c>
       <c s="12" r="E19">
-        <v>1635.000000</v>
+        <v>1600.000000</v>
       </c>
       <c s="12" r="F19">
-        <v>1643.000000</v>
+        <v>1625.000000</v>
       </c>
       <c s="12" r="H19">
-        <v>1640.000000</v>
+        <v>1620.000000</v>
       </c>
       <c s="13" r="I19">
-        <v>2967.000000</v>
+        <v>1490.000000</v>
       </c>
       <c s="12" r="J19">
-        <v>1638.000000</v>
+        <v>1625.000000</v>
       </c>
       <c s="14" r="K19">
-        <v>0.61</v>
+        <v>0.37</v>
       </c>
       <c s="13" r="L19">
-        <v>40488.000000</v>
+        <v>48077.000000</v>
       </c>
       <c s="13" r="M19">
-        <v>2368</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" ht="14.2" customHeight="0">
@@ -1142,34 +1142,34 @@
         </is>
       </c>
       <c s="11" r="C20">
-        <v>1658.000000</v>
+        <v>1649.000000</v>
       </c>
       <c s="12" r="D20">
-        <v>1675.000000</v>
+        <v>1645.000000</v>
       </c>
       <c s="12" r="E20">
-        <v>1673.000000</v>
+        <v>1645.000000</v>
       </c>
       <c s="12" r="F20">
-        <v>1675.000000</v>
+        <v>1645.000000</v>
       </c>
       <c s="12" r="H20">
-        <v>1673.000000</v>
+        <v>1645.000000</v>
       </c>
       <c s="13" r="I20">
-        <v>281.000000</v>
+        <v>1.000000</v>
       </c>
       <c s="12" r="J20">
-        <v>1668.000000</v>
+        <v>1655.000000</v>
       </c>
       <c s="14" r="K20">
-        <v>0.60</v>
+        <v>0.36</v>
       </c>
       <c s="13" r="L20">
         <v>1205.000000</v>
       </c>
       <c s="13" r="M20">
-        <v>280</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" ht="14.15" customHeight="0">
@@ -1184,34 +1184,34 @@
         </is>
       </c>
       <c s="11" r="C21">
-        <v>1688.000000</v>
+        <v>1679.000000</v>
       </c>
       <c s="12" r="D21">
-        <v>1685.500000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="E21">
-        <v>1685.500000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="F21">
-        <v>1685.500000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="H21">
-        <v>1685.500000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="I21">
-        <v>400.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="12" r="J21">
-        <v>1698.000000</v>
+        <v>1685.000000</v>
       </c>
       <c s="14" r="K21">
-        <v>0.59</v>
+        <v>0.36</v>
       </c>
       <c s="13" r="L21">
         <v>739.000000</v>
       </c>
       <c s="13" r="M21">
-        <v>160</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="14.15" customHeight="0">
@@ -1226,34 +1226,34 @@
         </is>
       </c>
       <c s="11" r="C22">
-        <v>1716.000000</v>
+        <v>1711.000000</v>
       </c>
       <c s="12" r="D22">
-        <v>1720.000000</v>
+        <v>1680.000000</v>
       </c>
       <c s="12" r="E22">
-        <v>1720.000000</v>
+        <v>1680.000000</v>
       </c>
       <c s="12" r="F22">
-        <v>1730.000000</v>
+        <v>1721.000000</v>
       </c>
       <c s="12" r="H22">
-        <v>1730.000000</v>
+        <v>1700.500000</v>
       </c>
       <c s="13" r="I22">
-        <v>130.000000</v>
+        <v>10106.000000</v>
       </c>
       <c s="12" r="J22">
-        <v>1730.000000</v>
+        <v>1717.000000</v>
       </c>
       <c s="14" r="K22">
-        <v>0.82</v>
+        <v>0.35</v>
       </c>
       <c s="13" r="L22">
-        <v>486.000000</v>
+        <v>595.000000</v>
       </c>
       <c s="13" r="M22">
-        <v>-30</v>
+        <v>-9899</v>
       </c>
     </row>
     <row r="23" ht="0.05" customHeight="1"/>
@@ -1402,10 +1402,10 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J27">
-        <v>19.142000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="K27">
-        <v>150.000000</v>
+        <v>1.000000</v>
       </c>
       <c s="13" r="L27">
         <v>0</v>
@@ -1441,7 +1441,7 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J28">
-        <v>2.791000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="K28">
         <v>500.000000</v>
@@ -1480,7 +1480,7 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J29">
-        <v>44.652000</v>
+        <v>27.982000</v>
       </c>
       <c s="13" r="K29">
         <v>275.000000</v>
@@ -1504,28 +1504,28 @@
         <v>1450.0000</v>
       </c>
       <c s="22" r="D30">
-        <v>12.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="E30">
-        <v>12.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="F30">
-        <v>12.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="H30">
-        <v>12.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="I30">
-        <v>450.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="J30">
-        <v>15.742000</v>
+        <v>7.143000</v>
       </c>
       <c s="13" r="K30">
         <v>450.000000</v>
       </c>
       <c s="13" r="L30">
-        <v>450</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="14.15" customHeight="0">
@@ -1543,28 +1543,28 @@
         <v>1460.0000</v>
       </c>
       <c s="22" r="D31">
-        <v>8.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="E31">
-        <v>8.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="F31">
-        <v>8.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="H31">
-        <v>8.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="13" r="I31">
-        <v>500.000000</v>
+        <v>0.000000</v>
       </c>
       <c s="22" r="J31">
-        <v>12.098000</v>
+        <v>5.063000</v>
       </c>
       <c s="13" r="K31">
         <v>500.000000</v>
       </c>
       <c s="13" r="L31">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="14.15" customHeight="0">
@@ -1721,107 +1721,107 @@
         </is>
       </c>
       <c s="26" r="B38">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c s="11" r="C38">
-        <v>1417.000000</v>
+        <v>1391.000000</v>
       </c>
       <c s="26" r="D38">
-        <v>46136</v>
+        <v>46141</v>
       </c>
       <c s="11" r="E38">
-        <v>1399.500000</v>
+        <v>1391.500000</v>
       </c>
       <c s="21" r="F38">
-        <v>1.25045</v>
+        <v>-0.03593</v>
       </c>
     </row>
     <row r="39" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A39">
         <is>
-          <t xml:space="preserve">Dólar BCRA A3500</t>
+          <t xml:space="preserve">Yuan CNH</t>
         </is>
       </c>
       <c s="26" r="B39">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c s="11" r="C39">
-        <v>1412.986500</v>
+        <v>202.121400</v>
       </c>
       <c s="26" r="D39">
-        <v>46136</v>
+        <v>46141</v>
       </c>
       <c s="11" r="E39">
-        <v>1397.206300</v>
+        <v>203.843200</v>
       </c>
       <c s="21" r="F39">
-        <v>1.12941</v>
+        <v>-0.84467</v>
       </c>
     </row>
     <row r="40" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A40">
         <is>
-          <t xml:space="preserve">Yuan CNH</t>
+          <t xml:space="preserve">Euro</t>
         </is>
       </c>
       <c s="26" r="B40">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c s="11" r="C40">
-        <v>206.970300</v>
+        <v>1616.158000</v>
       </c>
       <c s="26" r="D40">
-        <v>46136</v>
+        <v>46141</v>
       </c>
       <c s="11" r="E40">
-        <v>204.455300</v>
+        <v>1633.322000</v>
       </c>
       <c s="21" r="F40">
-        <v>1.23010</v>
+        <v>-1.05086</v>
       </c>
     </row>
     <row r="41" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A41">
         <is>
-          <t xml:space="preserve">Dólar BNA</t>
+          <t xml:space="preserve">Dólar BCRA A3500</t>
         </is>
       </c>
       <c s="26" r="B41">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c s="11" r="C41">
-        <v>1412.500000</v>
+        <v>1381.095400</v>
       </c>
       <c s="26" r="D41">
-        <v>46136</v>
+        <v>46141</v>
       </c>
       <c s="11" r="E41">
-        <v>1395.000000</v>
+        <v>1395.286600</v>
       </c>
       <c s="21" r="F41">
-        <v>1.25448</v>
+        <v>-1.01708</v>
       </c>
     </row>
     <row r="42" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A42">
         <is>
-          <t xml:space="preserve">Euro</t>
+          <t xml:space="preserve">Dólar BNA</t>
         </is>
       </c>
       <c s="26" r="B42">
-        <v>46139</v>
+        <v>46142</v>
       </c>
       <c s="11" r="C42">
-        <v>1660.118000</v>
+        <v>1386.500000</v>
       </c>
       <c s="26" r="D42">
-        <v>46136</v>
+        <v>46141</v>
       </c>
       <c s="11" r="E42">
-        <v>1636.408000</v>
+        <v>1387.000000</v>
       </c>
       <c s="21" r="F42">
-        <v>1.44891</v>
+        <v>-0.03605</v>
       </c>
     </row>
     <row r="43" ht="14.15" customHeight="0">

</xml_diff>

<commit_message>
refactor term structure analysis model
</commit_message>
<xml_diff>
--- a/usd-futures-curve-analyzer-matba-rofex/close.xlsx
+++ b/usd-futures-curve-analyzer-matba-rofex/close.xlsx
@@ -487,7 +487,7 @@
     <row r="6" ht="17.95" customHeight="1">
       <c s="4" t="inlineStr" r="A6">
         <is>
-          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : jueves, 30 de abril de 2026</t>
+          <t xml:space="preserve">Cierre Parcial A3 Mercados – Monedas : viernes, 15 de mayo de 2026</t>
         </is>
       </c>
     </row>
@@ -681,43 +681,43 @@
     <row r="11" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A11">
         <is>
-          <t xml:space="preserve">DLR042026</t>
+          <t xml:space="preserve">DLR052026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B11">
         <is>
-          <t xml:space="preserve">30/4/2026</t>
+          <t xml:space="preserve">29/5/2026</t>
         </is>
       </c>
       <c s="11" r="C11">
-        <v>1391.500000</v>
+        <v>1401.500000</v>
       </c>
       <c s="12" r="D11">
-        <v>1390.000000</v>
+        <v>1405.000000</v>
       </c>
       <c s="12" r="E11">
-        <v>1377.000000</v>
+        <v>1402.500000</v>
       </c>
       <c s="12" r="F11">
-        <v>1390.000000</v>
+        <v>1408.000000</v>
       </c>
       <c s="12" r="H11">
-        <v>1381.000000</v>
+        <v>1405.500000</v>
       </c>
       <c s="13" r="I11">
-        <v>880372.000000</v>
+        <v>580297.000000</v>
       </c>
       <c s="12" r="J11">
-        <v>1381.095400</v>
+        <v>1405.500000</v>
       </c>
       <c s="14" r="K11">
-        <v>-0.75</v>
+        <v>0.29</v>
       </c>
       <c s="13" r="L11">
-        <v>879270.000000</v>
+        <v>2385548.000000</v>
       </c>
       <c s="13" r="M11">
-        <v>-24712</v>
+        <v>-79975</v>
       </c>
       <c s="9" t="inlineStr" r="P11">
         <is>
@@ -733,7 +733,7 @@
         <v>0.000000</v>
       </c>
       <c s="13" r="S11">
-        <v>1726.000000</v>
+        <v>780.000000</v>
       </c>
       <c s="13" r="T11">
         <v>0.000000</v>
@@ -748,43 +748,43 @@
     <row r="12" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A12">
         <is>
-          <t xml:space="preserve">DLR052026</t>
+          <t xml:space="preserve">DLR062026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B12">
         <is>
-          <t xml:space="preserve">29/5/2026</t>
+          <t xml:space="preserve">30/6/2026</t>
         </is>
       </c>
       <c s="11" r="C12">
-        <v>1413.500000</v>
+        <v>1426.500000</v>
       </c>
       <c s="12" r="D12">
-        <v>1409.000000</v>
+        <v>1428.000000</v>
       </c>
       <c s="12" r="E12">
-        <v>1402.000000</v>
+        <v>1427.500000</v>
       </c>
       <c s="12" r="F12">
-        <v>1418.500000</v>
+        <v>1434.000000</v>
       </c>
       <c s="12" r="H12">
-        <v>1415.500000</v>
+        <v>1431.000000</v>
       </c>
       <c s="13" r="I12">
-        <v>822988.000000</v>
+        <v>221020.000000</v>
       </c>
       <c s="12" r="J12">
-        <v>1416.000000</v>
+        <v>1431.000000</v>
       </c>
       <c s="14" r="K12">
-        <v>0.18</v>
+        <v>0.32</v>
       </c>
       <c s="13" r="L12">
-        <v>2939947.000000</v>
+        <v>774361.000000</v>
       </c>
       <c s="13" r="M12">
-        <v>81820</v>
+        <v>-18456</v>
       </c>
       <c s="9" t="inlineStr" r="P12">
         <is>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c s="13" r="R12">
-        <v>1974201.000000</v>
+        <v>954409.000000</v>
       </c>
       <c s="13" r="S12">
-        <v>5199984.000000</v>
+        <v>4300999.000000</v>
       </c>
       <c s="13" r="T12">
-        <v>1974201000.000000</v>
+        <v>954409000.000000</v>
       </c>
       <c s="8" t="str" r="U12"/>
       <c s="9" t="inlineStr" r="V12">
@@ -815,43 +815,43 @@
     <row r="13" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A13">
         <is>
-          <t xml:space="preserve">DLR062026</t>
+          <t xml:space="preserve">DLR072026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B13">
         <is>
-          <t xml:space="preserve">30/6/2026</t>
+          <t xml:space="preserve">31/7/2026</t>
         </is>
       </c>
       <c s="11" r="C13">
-        <v>1440.000000</v>
+        <v>1455.500000</v>
       </c>
       <c s="12" r="D13">
-        <v>1434.000000</v>
+        <v>1459.000000</v>
       </c>
       <c s="12" r="E13">
-        <v>1428.000000</v>
+        <v>1456.500000</v>
       </c>
       <c s="12" r="F13">
-        <v>1447.000000</v>
+        <v>1463.000000</v>
       </c>
       <c s="12" r="H13">
-        <v>1443.000000</v>
+        <v>1460.500000</v>
       </c>
       <c s="13" r="I13">
-        <v>190696.000000</v>
+        <v>23946.000000</v>
       </c>
       <c s="12" r="J13">
-        <v>1443.500000</v>
+        <v>1460.500000</v>
       </c>
       <c s="14" r="K13">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c s="13" r="L13">
-        <v>592327.000000</v>
+        <v>482705.000000</v>
       </c>
       <c s="13" r="M13">
-        <v>26153</v>
+        <v>-2067</v>
       </c>
       <c s="16" t="inlineStr" r="P13">
         <is>
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c s="18" r="R13">
-        <v>1974201.000000</v>
+        <v>954409.000000</v>
       </c>
       <c s="18" r="S13">
-        <v>5201710.000000</v>
+        <v>4301779.000000</v>
       </c>
       <c s="18" r="T13">
-        <v>1974201000.000000</v>
+        <v>954409000.000000</v>
       </c>
       <c s="19" t="inlineStr" r="V13">
         <is>
@@ -881,510 +881,545 @@
     <row r="14" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A14">
         <is>
-          <t xml:space="preserve">DLR072026</t>
+          <t xml:space="preserve">DLR082026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B14">
         <is>
-          <t xml:space="preserve">31/7/2026</t>
+          <t xml:space="preserve">31/8/2026</t>
         </is>
       </c>
       <c s="11" r="C14">
-        <v>1470.000000</v>
+        <v>1485.500000</v>
       </c>
       <c s="12" r="D14">
-        <v>1461.500000</v>
+        <v>1490.000000</v>
       </c>
       <c s="12" r="E14">
-        <v>1458.500000</v>
+        <v>1490.000000</v>
       </c>
       <c s="12" r="F14">
-        <v>1476.500000</v>
+        <v>1495.000000</v>
       </c>
       <c s="12" r="H14">
-        <v>1470.500000</v>
+        <v>1492.500000</v>
       </c>
       <c s="13" r="I14">
-        <v>54466.000000</v>
+        <v>10566.000000</v>
       </c>
       <c s="12" r="J14">
-        <v>1474.000000</v>
+        <v>1491.500000</v>
       </c>
       <c s="14" r="K14">
-        <v>0.27</v>
+        <v>0.40</v>
       </c>
       <c s="13" r="L14">
-        <v>408191.000000</v>
+        <v>117894.000000</v>
       </c>
       <c s="13" r="M14">
-        <v>6609</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="15" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A15">
         <is>
-          <t xml:space="preserve">DLR082026</t>
+          <t xml:space="preserve">DLR092026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B15">
         <is>
-          <t xml:space="preserve">31/8/2026</t>
+          <t xml:space="preserve">30/9/2026</t>
         </is>
       </c>
       <c s="11" r="C15">
-        <v>1499.500000</v>
+        <v>1516.000000</v>
       </c>
       <c s="12" r="D15">
-        <v>1490.000000</v>
+        <v>1516.000000</v>
       </c>
       <c s="12" r="E15">
-        <v>1489.000000</v>
+        <v>1516.000000</v>
       </c>
       <c s="12" r="F15">
-        <v>1505.500000</v>
+        <v>1524.500000</v>
       </c>
       <c s="12" r="H15">
-        <v>1501.000000</v>
+        <v>1520.500000</v>
       </c>
       <c s="13" r="I15">
-        <v>2273.000000</v>
+        <v>32618.000000</v>
       </c>
       <c s="12" r="J15">
-        <v>1504.000000</v>
+        <v>1521.500000</v>
       </c>
       <c s="14" r="K15">
-        <v>0.30</v>
+        <v>0.36</v>
       </c>
       <c s="13" r="L15">
-        <v>106974.000000</v>
+        <v>146881.000000</v>
       </c>
       <c s="13" r="M15">
-        <v>2241</v>
+        <v>13506</v>
       </c>
     </row>
     <row r="16" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A16">
         <is>
-          <t xml:space="preserve">DLR092026</t>
+          <t xml:space="preserve">DLR102026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B16">
         <is>
-          <t xml:space="preserve">30/9/2026</t>
+          <t xml:space="preserve">30/10/2026</t>
         </is>
       </c>
       <c s="11" r="C16">
-        <v>1530.000000</v>
+        <v>1547.500000</v>
       </c>
       <c s="12" r="D16">
-        <v>1520.000000</v>
+        <v>1547.000000</v>
       </c>
       <c s="12" r="E16">
-        <v>1520.000000</v>
+        <v>1547.000000</v>
       </c>
       <c s="12" r="F16">
-        <v>1552.000000</v>
+        <v>1558.000000</v>
       </c>
       <c s="12" r="H16">
-        <v>1535.000000</v>
+        <v>1554.000000</v>
       </c>
       <c s="13" r="I16">
-        <v>7258.000000</v>
+        <v>33010.000000</v>
       </c>
       <c s="12" r="J16">
-        <v>1535.000000</v>
+        <v>1554.000000</v>
       </c>
       <c s="14" r="K16">
-        <v>0.33</v>
+        <v>0.42</v>
       </c>
       <c s="13" r="L16">
-        <v>79122.000000</v>
+        <v>108557.000000</v>
       </c>
       <c s="13" r="M16">
-        <v>-330</v>
+        <v>958</v>
       </c>
     </row>
     <row r="17" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A17">
         <is>
-          <t xml:space="preserve">DLR102026</t>
+          <t xml:space="preserve">DLR112026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B17">
         <is>
-          <t xml:space="preserve">30/10/2026</t>
+          <t xml:space="preserve">30/11/2026</t>
         </is>
       </c>
       <c s="11" r="C17">
-        <v>1560.000000</v>
+        <v>1580.000000</v>
       </c>
       <c s="12" r="D17">
-        <v>1550.000000</v>
+        <v>1588.000000</v>
       </c>
       <c s="12" r="E17">
-        <v>1550.000000</v>
+        <v>1588.000000</v>
       </c>
       <c s="12" r="F17">
-        <v>1564.500000</v>
+        <v>1588.000000</v>
       </c>
       <c s="12" r="H17">
-        <v>1564.500000</v>
+        <v>1588.000000</v>
       </c>
       <c s="13" r="I17">
-        <v>4549.000000</v>
+        <v>2000.000000</v>
       </c>
       <c s="12" r="J17">
-        <v>1564.500000</v>
+        <v>1588.000000</v>
       </c>
       <c s="14" r="K17">
-        <v>0.29</v>
+        <v>0.51</v>
       </c>
       <c s="13" r="L17">
-        <v>96152.000000</v>
+        <v>68601.000000</v>
       </c>
       <c s="13" r="M17">
-        <v>2556</v>
+        <v>994</v>
       </c>
     </row>
     <row r="18" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A18">
         <is>
-          <t xml:space="preserve">DLR112026</t>
+          <t xml:space="preserve">DLR122026</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B18">
         <is>
-          <t xml:space="preserve">30/11/2026</t>
+          <t xml:space="preserve">30/12/2026</t>
         </is>
       </c>
       <c s="11" r="C18">
-        <v>1589.000000</v>
+        <v>1617.000000</v>
       </c>
       <c s="12" r="D18">
-        <v>1590.000000</v>
+        <v>1618.500000</v>
       </c>
       <c s="12" r="E18">
-        <v>1590.000000</v>
+        <v>1618.500000</v>
       </c>
       <c s="12" r="F18">
-        <v>1600.000000</v>
+        <v>1625.500000</v>
       </c>
       <c s="12" r="H18">
-        <v>1600.000000</v>
+        <v>1623.000000</v>
       </c>
       <c s="13" r="I18">
-        <v>2.000000</v>
+        <v>12493.000000</v>
       </c>
       <c s="12" r="J18">
-        <v>1594.500000</v>
+        <v>1623.000000</v>
       </c>
       <c s="14" r="K18">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
       <c s="13" r="L18">
-        <v>47385.000000</v>
+        <v>107007.000000</v>
       </c>
       <c s="13" r="M18">
-        <v>-1</v>
+        <v>-465</v>
       </c>
     </row>
     <row r="19" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A19">
         <is>
-          <t xml:space="preserve">DLR122026</t>
+          <t xml:space="preserve">DLR012027</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B19">
         <is>
-          <t xml:space="preserve">30/12/2026</t>
+          <t xml:space="preserve">29/1/2027</t>
         </is>
       </c>
       <c s="11" r="C19">
-        <v>1619.000000</v>
+        <v>1652.000000</v>
       </c>
       <c s="12" r="D19">
-        <v>1600.000000</v>
+        <v>1650.000000</v>
       </c>
       <c s="12" r="E19">
-        <v>1600.000000</v>
+        <v>1650.000000</v>
       </c>
       <c s="12" r="F19">
-        <v>1625.000000</v>
+        <v>1660.000000</v>
       </c>
       <c s="12" r="H19">
-        <v>1620.000000</v>
+        <v>1656.500000</v>
       </c>
       <c s="13" r="I19">
-        <v>1490.000000</v>
+        <v>30950.000000</v>
       </c>
       <c s="12" r="J19">
-        <v>1625.000000</v>
+        <v>1657.500000</v>
       </c>
       <c s="14" r="K19">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c s="13" r="L19">
-        <v>48077.000000</v>
+        <v>33044.000000</v>
       </c>
       <c s="13" r="M19">
-        <v>262</v>
+        <v>23323</v>
       </c>
     </row>
     <row r="20" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A20">
         <is>
-          <t xml:space="preserve">DLR012027</t>
+          <t xml:space="preserve">DLR022027</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B20">
         <is>
-          <t xml:space="preserve">29/1/2027</t>
+          <t xml:space="preserve">26/2/2027</t>
         </is>
       </c>
       <c s="11" r="C20">
-        <v>1649.000000</v>
+        <v>1689.000000</v>
       </c>
       <c s="12" r="D20">
-        <v>1645.000000</v>
+        <v>1696.000000</v>
       </c>
       <c s="12" r="E20">
-        <v>1645.000000</v>
+        <v>1695.000000</v>
       </c>
       <c s="12" r="F20">
-        <v>1645.000000</v>
+        <v>1697.000000</v>
       </c>
       <c s="12" r="H20">
-        <v>1645.000000</v>
+        <v>1695.000000</v>
       </c>
       <c s="13" r="I20">
-        <v>1.000000</v>
+        <v>5000.000000</v>
       </c>
       <c s="12" r="J20">
-        <v>1655.000000</v>
+        <v>1694.500000</v>
       </c>
       <c s="14" r="K20">
-        <v>0.36</v>
+        <v>0.33</v>
       </c>
       <c s="13" r="L20">
-        <v>1205.000000</v>
+        <v>13335.000000</v>
       </c>
       <c s="13" r="M20">
-        <v>1</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="21" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A21">
         <is>
-          <t xml:space="preserve">DLR022027</t>
+          <t xml:space="preserve">DLR032027</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B21">
         <is>
-          <t xml:space="preserve">26/2/2027</t>
+          <t xml:space="preserve">31/3/2027</t>
         </is>
       </c>
       <c s="11" r="C21">
-        <v>1679.000000</v>
+        <v>1726.500000</v>
       </c>
       <c s="12" r="D21">
-        <v>0.000000</v>
+        <v>1730.000000</v>
       </c>
       <c s="12" r="E21">
-        <v>0.000000</v>
+        <v>1730.000000</v>
       </c>
       <c s="12" r="F21">
-        <v>0.000000</v>
+        <v>1739.000000</v>
       </c>
       <c s="12" r="H21">
-        <v>0.000000</v>
+        <v>1730.500000</v>
       </c>
       <c s="13" r="I21">
-        <v>0.000000</v>
+        <v>2509.000000</v>
       </c>
       <c s="12" r="J21">
-        <v>1685.000000</v>
+        <v>1732.000000</v>
       </c>
       <c s="14" r="K21">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c s="13" r="L21">
-        <v>739.000000</v>
+        <v>63066.000000</v>
       </c>
       <c s="13" r="M21">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="22" ht="41.4" customHeight="1"/>
+    <row r="23" ht="14.15" customHeight="0">
+      <c s="5" t="inlineStr" r="A23">
+        <is>
+          <t xml:space="preserve">Call</t>
+        </is>
+      </c>
+      <c s="5" t="inlineStr" r="B23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="H23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="I23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="J23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="K23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="L23">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14.2" customHeight="0">
+      <c s="20" t="inlineStr" r="A24">
+        <is>
+          <t xml:space="preserve">Posición</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="B24">
+        <is>
+          <t xml:space="preserve">Último Día Neg.</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="C24">
+        <is>
+          <t xml:space="preserve">Ejercicio</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="D24">
+        <is>
+          <t xml:space="preserve">Apertura</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="E24">
+        <is>
+          <t xml:space="preserve">Mín.</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="F24">
+        <is>
+          <t xml:space="preserve">Máx.</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="H24">
+        <is>
+          <t xml:space="preserve">Último</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="I24">
+        <is>
+          <t xml:space="preserve">Vol.</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="J24">
+        <is>
+          <t xml:space="preserve">Prima Ref. **</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="K24">
+        <is>
+          <t xml:space="preserve">I. A.*</t>
+        </is>
+      </c>
+      <c s="20" t="inlineStr" r="L24">
+        <is>
+          <t xml:space="preserve">Var. I.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A25">
+        <is>
+          <t xml:space="preserve">DLR052026 Call 1400</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B25">
+        <is>
+          <t xml:space="preserve">29/5/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C25">
+        <v>1400.0000</v>
+      </c>
+      <c s="22" r="D25">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E25">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F25">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H25">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I25">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J25">
+        <v>16.169000</v>
+      </c>
+      <c s="13" r="K25">
+        <v>475.000000</v>
+      </c>
+      <c s="13" r="L25">
         <v>0</v>
       </c>
     </row>
-    <row r="22" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A22">
-        <is>
-          <t xml:space="preserve">DLR032027</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B22">
-        <is>
-          <t xml:space="preserve">31/3/2027</t>
-        </is>
-      </c>
-      <c s="11" r="C22">
-        <v>1711.000000</v>
-      </c>
-      <c s="12" r="D22">
-        <v>1680.000000</v>
-      </c>
-      <c s="12" r="E22">
-        <v>1680.000000</v>
-      </c>
-      <c s="12" r="F22">
-        <v>1721.000000</v>
-      </c>
-      <c s="12" r="H22">
-        <v>1700.500000</v>
-      </c>
-      <c s="13" r="I22">
-        <v>10106.000000</v>
-      </c>
-      <c s="12" r="J22">
-        <v>1717.000000</v>
-      </c>
-      <c s="14" r="K22">
-        <v>0.35</v>
-      </c>
-      <c s="13" r="L22">
-        <v>595.000000</v>
-      </c>
-      <c s="13" r="M22">
-        <v>-9899</v>
-      </c>
-    </row>
-    <row r="23" ht="0.05" customHeight="1"/>
-    <row r="24" ht="41.4" customHeight="1"/>
-    <row r="25" ht="14.15" customHeight="0">
-      <c s="5" t="inlineStr" r="A25">
-        <is>
-          <t xml:space="preserve">Call</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="B25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="H25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="I25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="J25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="K25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="L25">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
     <row r="26" ht="14.2" customHeight="0">
-      <c s="20" t="inlineStr" r="A26">
-        <is>
-          <t xml:space="preserve">Posición</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="B26">
-        <is>
-          <t xml:space="preserve">Último Día Neg.</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="C26">
-        <is>
-          <t xml:space="preserve">Ejercicio</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="D26">
-        <is>
-          <t xml:space="preserve">Apertura</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="E26">
-        <is>
-          <t xml:space="preserve">Mín.</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="F26">
-        <is>
-          <t xml:space="preserve">Máx.</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="H26">
-        <is>
-          <t xml:space="preserve">Último</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="I26">
-        <is>
-          <t xml:space="preserve">Vol.</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="J26">
-        <is>
-          <t xml:space="preserve">Prima Ref. **</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="K26">
-        <is>
-          <t xml:space="preserve">I. A.*</t>
-        </is>
-      </c>
-      <c s="20" t="inlineStr" r="L26">
-        <is>
-          <t xml:space="preserve">Var. I.A.</t>
-        </is>
+      <c s="9" t="inlineStr" r="A26">
+        <is>
+          <t xml:space="preserve">DLR052026 Call 1410</t>
+        </is>
+      </c>
+      <c s="10" t="inlineStr" r="B26">
+        <is>
+          <t xml:space="preserve">29/5/2026</t>
+        </is>
+      </c>
+      <c s="21" r="C26">
+        <v>1410.0000</v>
+      </c>
+      <c s="22" r="D26">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="E26">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="F26">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="H26">
+        <v>0.000000</v>
+      </c>
+      <c s="13" r="I26">
+        <v>0.000000</v>
+      </c>
+      <c s="22" r="J26">
+        <v>11.199000</v>
+      </c>
+      <c s="13" r="K26">
+        <v>205.000000</v>
+      </c>
+      <c s="13" r="L26">
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="14.15" customHeight="0">
       <c s="9" t="inlineStr" r="A27">
         <is>
-          <t xml:space="preserve">DLR042026 Call 1400</t>
+          <t xml:space="preserve">DLR052026 Call 1450</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B27">
         <is>
-          <t xml:space="preserve">30/4/2026</t>
+          <t xml:space="preserve">29/5/2026</t>
         </is>
       </c>
       <c s="21" r="C27">
-        <v>1400.0000</v>
+        <v>1450.0000</v>
       </c>
       <c s="22" r="D27">
         <v>0.000000</v>
@@ -1402,10 +1437,10 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J27">
-        <v>0.000000</v>
+        <v>1.528000</v>
       </c>
       <c s="13" r="K27">
-        <v>1.000000</v>
+        <v>50.000000</v>
       </c>
       <c s="13" r="L27">
         <v>0</v>
@@ -1414,16 +1449,16 @@
     <row r="28" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A28">
         <is>
-          <t xml:space="preserve">DLR042026 Call 1430</t>
+          <t xml:space="preserve">DLR052026 Call 1460</t>
         </is>
       </c>
       <c s="10" t="inlineStr" r="B28">
         <is>
-          <t xml:space="preserve">30/4/2026</t>
+          <t xml:space="preserve">29/5/2026</t>
         </is>
       </c>
       <c s="21" r="C28">
-        <v>1430.0000</v>
+        <v>1460.0000</v>
       </c>
       <c s="22" r="D28">
         <v>0.000000</v>
@@ -1441,444 +1476,326 @@
         <v>0.000000</v>
       </c>
       <c s="22" r="J28">
-        <v>0.000000</v>
+        <v>0.805000</v>
       </c>
       <c s="13" r="K28">
-        <v>500.000000</v>
+        <v>50.000000</v>
       </c>
       <c s="13" r="L28">
         <v>0</v>
       </c>
     </row>
     <row r="29" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A29">
-        <is>
-          <t xml:space="preserve">DLR052026 Call 1400</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B29">
-        <is>
-          <t xml:space="preserve">29/5/2026</t>
-        </is>
-      </c>
-      <c s="21" r="C29">
-        <v>1400.0000</v>
-      </c>
-      <c s="22" r="D29">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="E29">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="F29">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="H29">
-        <v>0.000000</v>
-      </c>
-      <c s="13" r="I29">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="J29">
-        <v>27.982000</v>
-      </c>
-      <c s="13" r="K29">
-        <v>275.000000</v>
-      </c>
-      <c s="13" r="L29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A30">
-        <is>
-          <t xml:space="preserve">DLR052026 Call 1450</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B30">
-        <is>
-          <t xml:space="preserve">29/5/2026</t>
-        </is>
-      </c>
-      <c s="21" r="C30">
-        <v>1450.0000</v>
-      </c>
-      <c s="22" r="D30">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="E30">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="F30">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="H30">
-        <v>0.000000</v>
-      </c>
-      <c s="13" r="I30">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="J30">
-        <v>7.143000</v>
-      </c>
-      <c s="13" r="K30">
-        <v>450.000000</v>
-      </c>
-      <c s="13" r="L30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A31">
-        <is>
-          <t xml:space="preserve">DLR052026 Call 1460</t>
-        </is>
-      </c>
-      <c s="10" t="inlineStr" r="B31">
-        <is>
-          <t xml:space="preserve">29/5/2026</t>
-        </is>
-      </c>
-      <c s="21" r="C31">
-        <v>1460.0000</v>
-      </c>
-      <c s="22" r="D31">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="E31">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="F31">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="H31">
-        <v>0.000000</v>
-      </c>
-      <c s="13" r="I31">
-        <v>0.000000</v>
-      </c>
-      <c s="22" r="J31">
-        <v>5.063000</v>
-      </c>
-      <c s="13" r="K31">
-        <v>500.000000</v>
-      </c>
-      <c s="13" r="L31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="14.15" customHeight="0">
-      <c s="6" t="inlineStr" r="A32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="B32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="H32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="I32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="J32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="K32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="L32">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="0.05" customHeight="1"/>
-    <row r="34" ht="28.3" customHeight="1"/>
-    <row r="35" ht="18" customHeight="0">
-      <c s="23" t="inlineStr" r="A35">
+      <c s="6" t="inlineStr" r="A29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="B29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="H29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="I29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="J29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="K29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="L29">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28.35" customHeight="1"/>
+    <row r="31" ht="18" customHeight="0">
+      <c s="23" t="inlineStr" r="A31">
         <is>
           <t xml:space="preserve">Cotizaciones Spot</t>
         </is>
       </c>
-      <c s="23" t="inlineStr" r="B35">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="C35">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="D35">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="E35">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="23" t="inlineStr" r="F35">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="0">
-      <c s="24" t="inlineStr" r="A36">
+      <c s="23" t="inlineStr" r="B31">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="C31">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="D31">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="E31">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="23" t="inlineStr" r="F31">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="0">
+      <c s="24" t="inlineStr" r="A32">
         <is>
           <t xml:space="preserve">Producto</t>
         </is>
       </c>
-      <c s="7" t="inlineStr" r="B36">
+      <c s="7" t="inlineStr" r="B32">
         <is>
           <t xml:space="preserve">Última</t>
         </is>
       </c>
-      <c s="8" t="str" r="C36"/>
-      <c s="7" t="inlineStr" r="D36">
+      <c s="8" t="str" r="C32"/>
+      <c s="7" t="inlineStr" r="D32">
         <is>
           <t xml:space="preserve">Anterior</t>
         </is>
       </c>
-      <c s="8" t="str" r="E36"/>
-      <c s="24" t="inlineStr" r="F36">
+      <c s="8" t="str" r="E32"/>
+      <c s="24" t="inlineStr" r="F32">
         <is>
           <t xml:space="preserve">Var.%</t>
         </is>
       </c>
     </row>
+    <row r="33" ht="14.15" customHeight="0">
+      <c s="25" t="inlineStr" r="A33">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="7" t="inlineStr" r="B33">
+        <is>
+          <t xml:space="preserve">Fecha</t>
+        </is>
+      </c>
+      <c s="7" t="inlineStr" r="C33">
+        <is>
+          <t xml:space="preserve">Cotización</t>
+        </is>
+      </c>
+      <c s="7" t="inlineStr" r="D33">
+        <is>
+          <t xml:space="preserve">Fecha</t>
+        </is>
+      </c>
+      <c s="7" t="inlineStr" r="E33">
+        <is>
+          <t xml:space="preserve">Cotización</t>
+        </is>
+      </c>
+      <c s="25" t="inlineStr" r="F33">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A34">
+        <is>
+          <t xml:space="preserve">Dólar UST ART 000</t>
+        </is>
+      </c>
+      <c s="26" r="B34">
+        <v>46157</v>
+      </c>
+      <c s="11" r="C34">
+        <v>1394.500000</v>
+      </c>
+      <c s="26" r="D34">
+        <v>46156</v>
+      </c>
+      <c s="11" r="E34">
+        <v>1391.000000</v>
+      </c>
+      <c s="21" r="F34">
+        <v>0.25162</v>
+      </c>
+    </row>
+    <row r="35" ht="14.15" customHeight="0">
+      <c s="9" t="inlineStr" r="A35">
+        <is>
+          <t xml:space="preserve">Yuan CNH</t>
+        </is>
+      </c>
+      <c s="26" r="B35">
+        <v>46157</v>
+      </c>
+      <c s="11" r="C35">
+        <v>204.779600</v>
+      </c>
+      <c s="26" r="D35">
+        <v>46156</v>
+      </c>
+      <c s="11" r="E35">
+        <v>205.309800</v>
+      </c>
+      <c s="21" r="F35">
+        <v>-0.25824</v>
+      </c>
+    </row>
+    <row r="36" ht="14.2" customHeight="0">
+      <c s="9" t="inlineStr" r="A36">
+        <is>
+          <t xml:space="preserve">Dólar BNA</t>
+        </is>
+      </c>
+      <c s="26" r="B36">
+        <v>46157</v>
+      </c>
+      <c s="11" r="C36">
+        <v>1390.000000</v>
+      </c>
+      <c s="26" r="D36">
+        <v>46156</v>
+      </c>
+      <c s="11" r="E36">
+        <v>1386.500000</v>
+      </c>
+      <c s="21" r="F36">
+        <v>0.25243</v>
+      </c>
+    </row>
     <row r="37" ht="14.15" customHeight="0">
-      <c s="25" t="inlineStr" r="A37">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="7" t="inlineStr" r="B37">
-        <is>
-          <t xml:space="preserve">Fecha</t>
-        </is>
-      </c>
-      <c s="7" t="inlineStr" r="C37">
-        <is>
-          <t xml:space="preserve">Cotización</t>
-        </is>
-      </c>
-      <c s="7" t="inlineStr" r="D37">
-        <is>
-          <t xml:space="preserve">Fecha</t>
-        </is>
-      </c>
-      <c s="7" t="inlineStr" r="E37">
-        <is>
-          <t xml:space="preserve">Cotización</t>
-        </is>
-      </c>
-      <c s="25" t="inlineStr" r="F37">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c s="9" t="inlineStr" r="A37">
+        <is>
+          <t xml:space="preserve">Euro</t>
+        </is>
+      </c>
+      <c s="26" r="B37">
+        <v>46157</v>
+      </c>
+      <c s="11" r="C37">
+        <v>1622.510000</v>
+      </c>
+      <c s="26" r="D37">
+        <v>46156</v>
+      </c>
+      <c s="11" r="E37">
+        <v>1630.360000</v>
+      </c>
+      <c s="21" r="F37">
+        <v>-0.48149</v>
       </c>
     </row>
     <row r="38" ht="14.2" customHeight="0">
       <c s="9" t="inlineStr" r="A38">
         <is>
-          <t xml:space="preserve">Dólar UST ART 000</t>
+          <t xml:space="preserve">Dólar BCRA A3500</t>
         </is>
       </c>
       <c s="26" r="B38">
-        <v>46142</v>
+        <v>46157</v>
       </c>
       <c s="11" r="C38">
-        <v>1391.000000</v>
+        <v>1395.347800</v>
       </c>
       <c s="26" r="D38">
-        <v>46141</v>
+        <v>46156</v>
       </c>
       <c s="11" r="E38">
-        <v>1391.500000</v>
+        <v>1393.232200</v>
       </c>
       <c s="21" r="F38">
-        <v>-0.03593</v>
+        <v>0.15185</v>
       </c>
     </row>
     <row r="39" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A39">
-        <is>
-          <t xml:space="preserve">Yuan CNH</t>
-        </is>
-      </c>
-      <c s="26" r="B39">
-        <v>46142</v>
-      </c>
-      <c s="11" r="C39">
-        <v>202.121400</v>
-      </c>
-      <c s="26" r="D39">
-        <v>46141</v>
-      </c>
-      <c s="11" r="E39">
-        <v>203.843200</v>
-      </c>
-      <c s="21" r="F39">
-        <v>-0.84467</v>
-      </c>
-    </row>
-    <row r="40" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A40">
-        <is>
-          <t xml:space="preserve">Euro</t>
-        </is>
-      </c>
-      <c s="26" r="B40">
-        <v>46142</v>
-      </c>
-      <c s="11" r="C40">
-        <v>1616.158000</v>
-      </c>
-      <c s="26" r="D40">
-        <v>46141</v>
-      </c>
-      <c s="11" r="E40">
-        <v>1633.322000</v>
-      </c>
-      <c s="21" r="F40">
-        <v>-1.05086</v>
-      </c>
-    </row>
-    <row r="41" ht="14.15" customHeight="0">
-      <c s="9" t="inlineStr" r="A41">
-        <is>
-          <t xml:space="preserve">Dólar BCRA A3500</t>
-        </is>
-      </c>
-      <c s="26" r="B41">
-        <v>46142</v>
-      </c>
-      <c s="11" r="C41">
-        <v>1381.095400</v>
-      </c>
-      <c s="26" r="D41">
-        <v>46141</v>
-      </c>
-      <c s="11" r="E41">
-        <v>1395.286600</v>
-      </c>
-      <c s="21" r="F41">
-        <v>-1.01708</v>
-      </c>
-    </row>
-    <row r="42" ht="14.2" customHeight="0">
-      <c s="9" t="inlineStr" r="A42">
-        <is>
-          <t xml:space="preserve">Dólar BNA</t>
-        </is>
-      </c>
-      <c s="26" r="B42">
-        <v>46142</v>
-      </c>
-      <c s="11" r="C42">
-        <v>1386.500000</v>
-      </c>
-      <c s="26" r="D42">
-        <v>46141</v>
-      </c>
-      <c s="11" r="E42">
-        <v>1387.000000</v>
-      </c>
-      <c s="21" r="F42">
-        <v>-0.03605</v>
-      </c>
-    </row>
-    <row r="43" ht="14.15" customHeight="0">
-      <c s="6" t="inlineStr" r="A43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="B43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="C43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="E43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="F43">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22.5" customHeight="1"/>
-    <row r="45" ht="18" customHeight="1">
-      <c s="27" t="inlineStr" r="A45">
+      <c s="6" t="inlineStr" r="A39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="B39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="C39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="D39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="E39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c s="6" t="inlineStr" r="F39">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22.5" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1">
+      <c s="27" t="inlineStr" r="A41">
         <is>
           <t xml:space="preserve">* Los valores de interés abierto pueden variar una vez que se realice el proceso del día.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c s="27" t="inlineStr" r="A46">
+    <row r="42" ht="18" customHeight="1">
+      <c s="27" t="inlineStr" r="A42">
         <is>
           <t xml:space="preserve">** Los valores indicativos de las primas se calculan en base a los parámetros del SARP® y son valores teóricos. Los mismos no afectan el cálculo de márgenes y diferencias.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="17.95" customHeight="1">
-      <c s="27" t="inlineStr" r="A47">
+    <row r="43" ht="17.95" customHeight="1">
+      <c s="27" t="inlineStr" r="A43">
         <is>
           <t xml:space="preserve">Aquellas posiciones que registran volumen pero no tienen valores en "Apertura", "Mínimo", "Máximo" y "Último" fueron operadas a través de pases.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="0.05" customHeight="1"/>
+    <row r="44" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A2:S2"/>
@@ -1889,11 +1806,11 @@
     <mergeCell ref="T11:U11"/>
     <mergeCell ref="T12:U12"/>
     <mergeCell ref="T13:U13"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="A45:Y45"/>
-    <mergeCell ref="A46:Y46"/>
-    <mergeCell ref="A47:Y47"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="A41:Y41"/>
+    <mergeCell ref="A42:Y42"/>
+    <mergeCell ref="A43:Y43"/>
   </mergeCells>
   <pageMargins left="0.984251968503937" right="0.984251968503937" top="0.984251968503937" bottom="0.984251968503937" header="0.984251968503937" footer="0.984251968503937"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>